<commit_message>
Horizontal bar charts, job names instead of codes, muted palette
- Categorical charts (jobs, engagements, grants) are horizontal bars,
  on the site and in the PDFs; label column sizes to the longest name
- Data labels smaller and quieter, with a white halo over the target line
- Jobs, engagements and grants are shown by name everywhere (codes kept
  only as database keys); NFP P&L lines drop the grant codes
- Muted palette: sage green on target, sand below target, dusty brick
  for very late/overdue, grey-blue for on its way; target line is a
  near-black dotted line instead of orange

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/nfp-sample-statements.xlsx
+++ b/media/exports/nfp-sample-statements.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Grants'!$A$4:$N$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Grants'!$A$4:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -619,7 +619,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Youth</t>
+          <t>Youth outreach</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
@@ -629,7 +629,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Housing</t>
+          <t>Housing support</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
@@ -639,7 +639,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Meals</t>
+          <t>Community meals</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
@@ -649,7 +649,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Digital</t>
+          <t>Digital literacy</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
@@ -659,7 +659,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mind</t>
+          <t>Mental health first aid</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
@@ -669,7 +669,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Volunteer</t>
+          <t>Volunteer coordinator</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
@@ -752,7 +752,7 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>G-101 Youth outreach grant</t>
+          <t>Youth outreach grant</t>
         </is>
       </c>
       <c r="B6" s="14" t="n">
@@ -769,7 +769,7 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>G-102 Housing support grant</t>
+          <t>Housing support grant</t>
         </is>
       </c>
       <c r="B7" s="14" t="n">
@@ -786,7 +786,7 @@
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>G-103 Community meals grant</t>
+          <t>Community meals grant</t>
         </is>
       </c>
       <c r="B8" s="14" t="n">
@@ -803,7 +803,7 @@
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>G-104 Digital literacy grant</t>
+          <t>Digital literacy grant</t>
         </is>
       </c>
       <c r="B9" s="14" t="n">
@@ -820,7 +820,7 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>G-105 Mental health first aid grant</t>
+          <t>Mental health first aid grant</t>
         </is>
       </c>
       <c r="B10" s="14" t="n">
@@ -837,7 +837,7 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>G-106 Volunteer coordinator grant</t>
+          <t>Volunteer coordinator grant</t>
         </is>
       </c>
       <c r="B11" s="14" t="n">
@@ -1815,12 +1815,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
@@ -1831,7 +1831,6 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1851,70 +1850,65 @@
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>Grant</t>
+          <t>Program</t>
         </is>
       </c>
       <c r="B4" s="20" t="inlineStr">
         <is>
-          <t>Program</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
           <t>Funder</t>
         </is>
       </c>
-      <c r="D4" s="21" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
+      <c r="D4" s="20" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
       <c r="E4" s="20" t="inlineStr">
         <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="inlineStr">
-        <is>
           <t>End</t>
         </is>
       </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Received to date</t>
+        </is>
+      </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>Received to date</t>
+          <t>Spent to date</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>Spent to date</t>
+          <t>Spent Aug</t>
         </is>
       </c>
       <c r="I4" s="21" t="inlineStr">
         <is>
-          <t>Spent Aug</t>
+          <t>Spent Sep</t>
         </is>
       </c>
       <c r="J4" s="21" t="inlineStr">
         <is>
-          <t>Spent Sep</t>
+          <t>Budget to date</t>
         </is>
       </c>
       <c r="K4" s="21" t="inlineStr">
         <is>
-          <t>Budget to date</t>
+          <t>Spend vs budget %</t>
         </is>
       </c>
       <c r="L4" s="21" t="inlineStr">
         <is>
-          <t>Spend vs budget %</t>
+          <t>Still to spend</t>
         </is>
       </c>
       <c r="M4" s="21" t="inlineStr">
-        <is>
-          <t>Still to spend</t>
-        </is>
-      </c>
-      <c r="N4" s="21" t="inlineStr">
         <is>
           <t>Months left</t>
         </is>
@@ -1923,329 +1917,299 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>G-101</t>
+          <t>Youth outreach</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Youth outreach</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
           <t>State Department of Families</t>
         </is>
       </c>
-      <c r="D5" s="22" t="n">
+      <c r="C5" s="22" t="n">
         <v>480000</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2025-07-01</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2025-07-01</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
           <t>2027-06-30</t>
         </is>
       </c>
+      <c r="F5" s="22" t="n">
+        <v>300000</v>
+      </c>
       <c r="G5" s="22" t="n">
+        <v>306300</v>
+      </c>
+      <c r="H5" s="22" t="n">
+        <v>21500</v>
+      </c>
+      <c r="I5" s="22" t="n">
+        <v>22800</v>
+      </c>
+      <c r="J5" s="22" t="n">
         <v>300000</v>
       </c>
-      <c r="H5" s="22" t="n">
-        <v>306300</v>
-      </c>
-      <c r="I5" s="22" t="n">
-        <v>21500</v>
-      </c>
-      <c r="J5" s="22" t="n">
-        <v>22800</v>
-      </c>
-      <c r="K5" s="22" t="n">
-        <v>300000</v>
-      </c>
-      <c r="L5" s="8" t="n">
+      <c r="K5" s="8" t="n">
         <v>102.1</v>
       </c>
+      <c r="L5" s="22" t="n">
+        <v>173700</v>
+      </c>
       <c r="M5" s="22" t="n">
-        <v>173700</v>
-      </c>
-      <c r="N5" s="22" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>G-102</t>
+          <t>Housing support</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Housing support</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
           <t>State Housing Program</t>
         </is>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="C6" s="22" t="n">
         <v>360000</v>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
           <t>2026-12-31</t>
         </is>
       </c>
+      <c r="F6" s="22" t="n">
+        <v>360000</v>
+      </c>
       <c r="G6" s="22" t="n">
-        <v>360000</v>
+        <v>257700</v>
       </c>
       <c r="H6" s="22" t="n">
-        <v>257700</v>
+        <v>30500</v>
       </c>
       <c r="I6" s="22" t="n">
-        <v>30500</v>
+        <v>31200</v>
       </c>
       <c r="J6" s="22" t="n">
-        <v>31200</v>
-      </c>
-      <c r="K6" s="22" t="n">
         <v>270000</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="K6" s="8" t="n">
         <v>95.40000000000001</v>
       </c>
+      <c r="L6" s="22" t="n">
+        <v>102300</v>
+      </c>
       <c r="M6" s="22" t="n">
-        <v>102300</v>
-      </c>
-      <c r="N6" s="22" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>G-103</t>
+          <t>Community meals</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Community meals</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
           <t>Local council community grant</t>
         </is>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="C7" s="22" t="n">
         <v>48000</v>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
           <t>2027-06-30</t>
         </is>
       </c>
+      <c r="F7" s="22" t="n">
+        <v>48000</v>
+      </c>
       <c r="G7" s="22" t="n">
-        <v>48000</v>
+        <v>12000</v>
       </c>
       <c r="H7" s="22" t="n">
+        <v>4100</v>
+      </c>
+      <c r="I7" s="22" t="n">
+        <v>4300</v>
+      </c>
+      <c r="J7" s="22" t="n">
         <v>12000</v>
       </c>
-      <c r="I7" s="22" t="n">
-        <v>4100</v>
-      </c>
-      <c r="J7" s="22" t="n">
-        <v>4300</v>
-      </c>
-      <c r="K7" s="22" t="n">
-        <v>12000</v>
-      </c>
-      <c r="L7" s="8" t="n">
+      <c r="K7" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="L7" s="22" t="n">
+        <v>36000</v>
+      </c>
       <c r="M7" s="22" t="n">
-        <v>36000</v>
-      </c>
-      <c r="N7" s="22" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>G-104</t>
+          <t>Digital literacy</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Digital literacy</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
           <t>Philanthropic foundation</t>
         </is>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="C8" s="22" t="n">
         <v>90000</v>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2025-10-01</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
           <t>2027-03-31</t>
         </is>
       </c>
+      <c r="F8" s="22" t="n">
+        <v>45000</v>
+      </c>
       <c r="G8" s="22" t="n">
-        <v>45000</v>
+        <v>59600</v>
       </c>
       <c r="H8" s="22" t="n">
-        <v>59600</v>
+        <v>5200</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>5200</v>
+        <v>4900</v>
       </c>
       <c r="J8" s="22" t="n">
-        <v>4900</v>
-      </c>
-      <c r="K8" s="22" t="n">
         <v>60000</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="K8" s="8" t="n">
         <v>99.3</v>
       </c>
+      <c r="L8" s="22" t="n">
+        <v>30400</v>
+      </c>
       <c r="M8" s="22" t="n">
-        <v>30400</v>
-      </c>
-      <c r="N8" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>G-105</t>
+          <t>Mental health first aid</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mental health first aid</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
           <t>Federal health program</t>
         </is>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="C9" s="22" t="n">
         <v>120000</v>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
           <t>2027-03-31</t>
         </is>
       </c>
+      <c r="F9" s="22" t="n">
+        <v>60000</v>
+      </c>
       <c r="G9" s="22" t="n">
+        <v>57200</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <v>9400</v>
+      </c>
+      <c r="I9" s="22" t="n">
+        <v>10800</v>
+      </c>
+      <c r="J9" s="22" t="n">
         <v>60000</v>
       </c>
-      <c r="H9" s="22" t="n">
-        <v>57200</v>
-      </c>
-      <c r="I9" s="22" t="n">
-        <v>9400</v>
-      </c>
-      <c r="J9" s="22" t="n">
-        <v>10800</v>
-      </c>
-      <c r="K9" s="22" t="n">
-        <v>60000</v>
-      </c>
-      <c r="L9" s="8" t="n">
+      <c r="K9" s="8" t="n">
         <v>95.3</v>
       </c>
+      <c r="L9" s="22" t="n">
+        <v>62800</v>
+      </c>
       <c r="M9" s="22" t="n">
-        <v>62800</v>
-      </c>
-      <c r="N9" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>G-106</t>
+          <t>Volunteer coordinator</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Volunteer coordinator</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
           <t>State volunteering grant</t>
         </is>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="C10" s="22" t="n">
         <v>36000</v>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
           <t>2027-02-28</t>
         </is>
       </c>
+      <c r="F10" s="22" t="n">
+        <v>36000</v>
+      </c>
       <c r="G10" s="22" t="n">
-        <v>36000</v>
+        <v>21000</v>
       </c>
       <c r="H10" s="22" t="n">
-        <v>21000</v>
+        <v>3000</v>
       </c>
       <c r="I10" s="22" t="n">
         <v>3000</v>
       </c>
       <c r="J10" s="22" t="n">
-        <v>3000</v>
-      </c>
-      <c r="K10" s="22" t="n">
         <v>21000</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="K10" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="L10" s="22" t="n">
+        <v>15000</v>
+      </c>
       <c r="M10" s="22" t="n">
-        <v>15000</v>
-      </c>
-      <c r="N10" s="22" t="n">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:N10"/>
+  <autoFilter ref="A4:M10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2330,7 +2294,7 @@
     <row r="10">
       <c r="A10" s="23" t="inlineStr">
         <is>
-          <t>G-101 Youth outreach</t>
+          <t>Youth outreach</t>
         </is>
       </c>
       <c r="B10" s="24" t="inlineStr">
@@ -2342,7 +2306,7 @@
     <row r="11">
       <c r="A11" s="23" t="inlineStr">
         <is>
-          <t>G-102 Housing support</t>
+          <t>Housing support</t>
         </is>
       </c>
       <c r="B11" s="24" t="inlineStr">
@@ -2354,7 +2318,7 @@
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>G-103 Community meals</t>
+          <t>Community meals</t>
         </is>
       </c>
       <c r="B12" s="24" t="inlineStr">
@@ -2366,7 +2330,7 @@
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
         <is>
-          <t>G-104 Digital literacy</t>
+          <t>Digital literacy</t>
         </is>
       </c>
       <c r="B13" s="24" t="inlineStr">
@@ -2378,7 +2342,7 @@
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
         <is>
-          <t>G-105 Mental health first aid</t>
+          <t>Mental health first aid</t>
         </is>
       </c>
       <c r="B14" s="24" t="inlineStr">
@@ -2390,7 +2354,7 @@
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
         <is>
-          <t>G-106 Volunteer coordinator</t>
+          <t>Volunteer coordinator</t>
         </is>
       </c>
       <c r="B15" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Workings behind every number; grants by program with %/$ toggle and spend over time
- Every headline number and every chart bar opens "How it's worked out":
  formula, September and August inputs, notes (e.g. cost to win a
  customer = marketing spend / new customers; technician time = job
  hours / technicians x working days x 7.6)
- Grants chart: one bar per program, total to date, plain colours;
  toggle between % of budget and $ spent (with a budget-to-date marker)
- Each grant opens its monthly spend since it started against the
  monthly budget (monthly history added to the model, checked to add
  up; new fact_grant_spend_month table)
- Workings sheet in each Excel download and a workings page in each PDF
- "cafe", not "café"

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/nfp-sample-statements.xlsx
+++ b/media/exports/nfp-sample-statements.xlsx
@@ -11,11 +11,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PandL" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance sheet" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash flow" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grants" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Grants" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Grants'!$A$4:$M$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Grants'!$A$4:$M$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -122,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -157,13 +158,20 @@
     <xf numFmtId="165" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" indent="1"/>
     </xf>
@@ -612,7 +620,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Grant spend vs budget to date (%)</t>
+          <t>Grant spend to date against budget</t>
         </is>
       </c>
     </row>
@@ -1810,6 +1818,1810 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C172"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How each number is worked out</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · generated 2026-10-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Cost to raise a dollar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Fundraising costs ÷ money raised (grants, donations, events)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="20" t="inlineStr"/>
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>Grant writing and reporting</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>$7,100</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>$7,100</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>Donor campaigns</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>$5,400</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
+        <is>
+          <t>$2,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>Event costs</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>$16,900</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
+        <is>
+          <t>$2,400</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>Fundraising costs</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="inlineStr">
+        <is>
+          <t>$29,400</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
+        <is>
+          <t>$11,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Grant income</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>$77,000</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
+        <is>
+          <t>$73,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Donations</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>$27,900</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
+        <is>
+          <t>$18,400</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>Fundraising events</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>$41,600</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
+        <is>
+          <t>$0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>Money raised</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>$146,500</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
+        <is>
+          <t>$92,100</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Cost per dollar raised</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>20¢</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
+        <is>
+          <t>13¢</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>September's gala raised $41,600 but cost $16,900 to run, which lifts the month's figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>Unrestricted cash runway</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>(Cash at bank − unspent grant money) ÷ this month's cash spending</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="20" t="inlineStr"/>
+      <c r="B21" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>Aug 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Cash at bank</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>$480,780</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>$525,675</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="21" t="inlineStr">
+        <is>
+          <t>Less unspent grant money (belongs to funders' programs)</t>
+        </is>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>$-156,100</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>$-221,900</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>Unrestricted cash</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>$324,680</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>$303,775</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>Cash spending in the month (expenses less depreciation)</t>
+        </is>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>$162,900</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>$141,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Runway</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>2.0 months</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>2.2 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Reserves target: 3 months.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Grants ending in the next 6 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Grant total − spent to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr"/>
+      <c r="B32" s="20" t="inlineStr">
+        <is>
+          <t>Ends</t>
+        </is>
+      </c>
+      <c r="C32" s="20" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="21" t="inlineStr">
+        <is>
+          <t>Housing support</t>
+        </is>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>31 Dec 2026</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>$102,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>28 Feb 2027</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t>$15,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="inlineStr"/>
+      <c r="C35" s="22" t="inlineStr">
+        <is>
+          <t>$117,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Unspent money usually has to be returned, or an extension negotiated, so plan the spending now.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Youth outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>State Department of Families · $480,000 · Jul 2025 to Jun 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="20" t="inlineStr"/>
+      <c r="B41" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="21" t="inlineStr">
+        <is>
+          <t>Received from the funder</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>$300,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="21" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>$173,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="21" t="inlineStr">
+        <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>$306,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>$300,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="21" t="inlineStr">
+        <is>
+          <t>Spent against budget</t>
+        </is>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>102.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Spend by month against budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B50" s="20" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Jul 25</t>
+        </is>
+      </c>
+      <c r="B51" s="23" t="n">
+        <v>17363</v>
+      </c>
+      <c r="C51" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Aug 25</t>
+        </is>
+      </c>
+      <c r="B52" s="23" t="n">
+        <v>21144</v>
+      </c>
+      <c r="C52" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Sep 25</t>
+        </is>
+      </c>
+      <c r="B53" s="23" t="n">
+        <v>17537</v>
+      </c>
+      <c r="C53" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Oct 25</t>
+        </is>
+      </c>
+      <c r="B54" s="23" t="n">
+        <v>21925</v>
+      </c>
+      <c r="C54" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Nov 25</t>
+        </is>
+      </c>
+      <c r="B55" s="23" t="n">
+        <v>21079</v>
+      </c>
+      <c r="C55" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Dec 25</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="n">
+        <v>19272</v>
+      </c>
+      <c r="C56" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Jan 26</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="n">
+        <v>21157</v>
+      </c>
+      <c r="C57" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Feb 26</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="n">
+        <v>20743</v>
+      </c>
+      <c r="C58" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Mar 26</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="n">
+        <v>16515</v>
+      </c>
+      <c r="C59" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Apr 26</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="n">
+        <v>20451</v>
+      </c>
+      <c r="C60" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>May 26</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="n">
+        <v>21174</v>
+      </c>
+      <c r="C61" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="n">
+        <v>20366</v>
+      </c>
+      <c r="C62" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B63" s="23" t="n">
+        <v>23274</v>
+      </c>
+      <c r="C63" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B64" s="23" t="n">
+        <v>21500</v>
+      </c>
+      <c r="C64" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B65" s="23" t="n">
+        <v>22800</v>
+      </c>
+      <c r="C65" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>Housing support</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>State Housing Program · $360,000 · Jan 2026 to Dec 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="20" t="inlineStr"/>
+      <c r="B70" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="21" t="inlineStr">
+        <is>
+          <t>Received from the funder</t>
+        </is>
+      </c>
+      <c r="B71" s="22" t="inlineStr">
+        <is>
+          <t>$360,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="21" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+      <c r="B72" s="22" t="inlineStr">
+        <is>
+          <t>$102,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="21" t="inlineStr">
+        <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B73" s="22" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B74" s="22" t="inlineStr">
+        <is>
+          <t>$257,700</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B75" s="22" t="inlineStr">
+        <is>
+          <t>$270,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="21" t="inlineStr">
+        <is>
+          <t>Spent against budget</t>
+        </is>
+      </c>
+      <c r="B76" s="22" t="inlineStr">
+        <is>
+          <t>95.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="7" t="inlineStr">
+        <is>
+          <t>Spend by month against budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B79" s="20" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C79" s="20" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Jan 26</t>
+        </is>
+      </c>
+      <c r="B80" s="23" t="n">
+        <v>30502</v>
+      </c>
+      <c r="C80" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Feb 26</t>
+        </is>
+      </c>
+      <c r="B81" s="23" t="n">
+        <v>26508</v>
+      </c>
+      <c r="C81" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Mar 26</t>
+        </is>
+      </c>
+      <c r="B82" s="23" t="n">
+        <v>24832</v>
+      </c>
+      <c r="C82" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Apr 26</t>
+        </is>
+      </c>
+      <c r="B83" s="23" t="n">
+        <v>23730</v>
+      </c>
+      <c r="C83" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>May 26</t>
+        </is>
+      </c>
+      <c r="B84" s="23" t="n">
+        <v>31337</v>
+      </c>
+      <c r="C84" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B85" s="23" t="n">
+        <v>29994</v>
+      </c>
+      <c r="C85" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B86" s="23" t="n">
+        <v>29097</v>
+      </c>
+      <c r="C86" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B87" s="23" t="n">
+        <v>30500</v>
+      </c>
+      <c r="C87" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B88" s="23" t="n">
+        <v>31200</v>
+      </c>
+      <c r="C88" s="23" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Community meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="9" t="inlineStr">
+        <is>
+          <t>Local council community grant · $48,000 · Jul 2026 to Jun 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="20" t="inlineStr"/>
+      <c r="B93" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="21" t="inlineStr">
+        <is>
+          <t>Received from the funder</t>
+        </is>
+      </c>
+      <c r="B94" s="22" t="inlineStr">
+        <is>
+          <t>$48,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="21" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+      <c r="B95" s="22" t="inlineStr">
+        <is>
+          <t>$36,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="21" t="inlineStr">
+        <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B96" s="22" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B97" s="22" t="inlineStr">
+        <is>
+          <t>$12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B98" s="22" t="inlineStr">
+        <is>
+          <t>$12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="21" t="inlineStr">
+        <is>
+          <t>Spent against budget</t>
+        </is>
+      </c>
+      <c r="B99" s="22" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t>Spend by month against budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B102" s="20" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C102" s="20" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B103" s="23" t="n">
+        <v>3600</v>
+      </c>
+      <c r="C103" s="23" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B104" s="23" t="n">
+        <v>4100</v>
+      </c>
+      <c r="C104" s="23" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B105" s="23" t="n">
+        <v>4300</v>
+      </c>
+      <c r="C105" s="23" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="4" t="inlineStr">
+        <is>
+          <t>Digital literacy</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="9" t="inlineStr">
+        <is>
+          <t>Philanthropic foundation · $90,000 · Oct 2025 to Mar 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="20" t="inlineStr"/>
+      <c r="B110" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="21" t="inlineStr">
+        <is>
+          <t>Received from the funder</t>
+        </is>
+      </c>
+      <c r="B111" s="22" t="inlineStr">
+        <is>
+          <t>$45,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="21" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+      <c r="B112" s="22" t="inlineStr">
+        <is>
+          <t>$30,400</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="21" t="inlineStr">
+        <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B113" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B114" s="22" t="inlineStr">
+        <is>
+          <t>$59,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B115" s="22" t="inlineStr">
+        <is>
+          <t>$60,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="21" t="inlineStr">
+        <is>
+          <t>Spent against budget</t>
+        </is>
+      </c>
+      <c r="B116" s="22" t="inlineStr">
+        <is>
+          <t>99.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>Spend by month against budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B119" s="20" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C119" s="20" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Oct 25</t>
+        </is>
+      </c>
+      <c r="B120" s="23" t="n">
+        <v>5160</v>
+      </c>
+      <c r="C120" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Nov 25</t>
+        </is>
+      </c>
+      <c r="B121" s="23" t="n">
+        <v>4585</v>
+      </c>
+      <c r="C121" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Dec 25</t>
+        </is>
+      </c>
+      <c r="B122" s="23" t="n">
+        <v>5221</v>
+      </c>
+      <c r="C122" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Jan 26</t>
+        </is>
+      </c>
+      <c r="B123" s="23" t="n">
+        <v>4426</v>
+      </c>
+      <c r="C123" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Feb 26</t>
+        </is>
+      </c>
+      <c r="B124" s="23" t="n">
+        <v>5408</v>
+      </c>
+      <c r="C124" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Mar 26</t>
+        </is>
+      </c>
+      <c r="B125" s="23" t="n">
+        <v>5427</v>
+      </c>
+      <c r="C125" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Apr 26</t>
+        </is>
+      </c>
+      <c r="B126" s="23" t="n">
+        <v>5509</v>
+      </c>
+      <c r="C126" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>May 26</t>
+        </is>
+      </c>
+      <c r="B127" s="23" t="n">
+        <v>4635</v>
+      </c>
+      <c r="C127" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B128" s="23" t="n">
+        <v>4316</v>
+      </c>
+      <c r="C128" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B129" s="23" t="n">
+        <v>4813</v>
+      </c>
+      <c r="C129" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B130" s="23" t="n">
+        <v>5200</v>
+      </c>
+      <c r="C130" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B131" s="23" t="n">
+        <v>4900</v>
+      </c>
+      <c r="C131" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="4" t="inlineStr">
+        <is>
+          <t>Mental health first aid</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="9" t="inlineStr">
+        <is>
+          <t>Federal health program · $120,000 · Apr 2026 to Mar 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="20" t="inlineStr"/>
+      <c r="B136" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="21" t="inlineStr">
+        <is>
+          <t>Received from the funder</t>
+        </is>
+      </c>
+      <c r="B137" s="22" t="inlineStr">
+        <is>
+          <t>$60,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="21" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+      <c r="B138" s="22" t="inlineStr">
+        <is>
+          <t>$62,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="21" t="inlineStr">
+        <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B139" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B140" s="22" t="inlineStr">
+        <is>
+          <t>$57,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B141" s="22" t="inlineStr">
+        <is>
+          <t>$60,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="21" t="inlineStr">
+        <is>
+          <t>Spent against budget</t>
+        </is>
+      </c>
+      <c r="B142" s="22" t="inlineStr">
+        <is>
+          <t>95.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="7" t="inlineStr">
+        <is>
+          <t>Spend by month against budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B145" s="20" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C145" s="20" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Apr 26</t>
+        </is>
+      </c>
+      <c r="B146" s="23" t="n">
+        <v>9584</v>
+      </c>
+      <c r="C146" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>May 26</t>
+        </is>
+      </c>
+      <c r="B147" s="23" t="n">
+        <v>8950</v>
+      </c>
+      <c r="C147" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B148" s="23" t="n">
+        <v>9797</v>
+      </c>
+      <c r="C148" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B149" s="23" t="n">
+        <v>8669</v>
+      </c>
+      <c r="C149" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B150" s="23" t="n">
+        <v>9400</v>
+      </c>
+      <c r="C150" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B151" s="23" t="n">
+        <v>10800</v>
+      </c>
+      <c r="C151" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>Volunteer coordinator</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="9" t="inlineStr">
+        <is>
+          <t>State volunteering grant · $36,000 · Mar 2026 to Feb 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="20" t="inlineStr"/>
+      <c r="B156" s="20" t="inlineStr">
+        <is>
+          <t>Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="21" t="inlineStr">
+        <is>
+          <t>Received from the funder</t>
+        </is>
+      </c>
+      <c r="B157" s="22" t="inlineStr">
+        <is>
+          <t>$36,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="21" t="inlineStr">
+        <is>
+          <t>Still to spend</t>
+        </is>
+      </c>
+      <c r="B158" s="22" t="inlineStr">
+        <is>
+          <t>$15,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="21" t="inlineStr">
+        <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B159" s="22" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B160" s="22" t="inlineStr">
+        <is>
+          <t>$21,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B161" s="22" t="inlineStr">
+        <is>
+          <t>$21,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="21" t="inlineStr">
+        <is>
+          <t>Spent against budget</t>
+        </is>
+      </c>
+      <c r="B162" s="22" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="7" t="inlineStr">
+        <is>
+          <t>Spend by month against budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="20" t="inlineStr">
+        <is>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B165" s="20" t="inlineStr">
+        <is>
+          <t>Spend</t>
+        </is>
+      </c>
+      <c r="C165" s="20" t="inlineStr">
+        <is>
+          <t>Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Mar 26</t>
+        </is>
+      </c>
+      <c r="B166" s="23" t="n">
+        <v>2932</v>
+      </c>
+      <c r="C166" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Apr 26</t>
+        </is>
+      </c>
+      <c r="B167" s="23" t="n">
+        <v>3555</v>
+      </c>
+      <c r="C167" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>May 26</t>
+        </is>
+      </c>
+      <c r="B168" s="23" t="n">
+        <v>2649</v>
+      </c>
+      <c r="C168" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B169" s="23" t="n">
+        <v>2699</v>
+      </c>
+      <c r="C169" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B170" s="23" t="n">
+        <v>3165</v>
+      </c>
+      <c r="C170" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B171" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C171" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B172" s="23" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C172" s="23" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1848,67 +3660,67 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Funder</t>
         </is>
       </c>
-      <c r="C4" s="21" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="F4" s="21" t="inlineStr">
+      <c r="F4" s="25" t="inlineStr">
         <is>
           <t>Received to date</t>
         </is>
       </c>
-      <c r="G4" s="21" t="inlineStr">
+      <c r="G4" s="25" t="inlineStr">
         <is>
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="H4" s="25" t="inlineStr">
         <is>
           <t>Spent Aug</t>
         </is>
       </c>
-      <c r="I4" s="21" t="inlineStr">
+      <c r="I4" s="25" t="inlineStr">
         <is>
           <t>Spent Sep</t>
         </is>
       </c>
-      <c r="J4" s="21" t="inlineStr">
+      <c r="J4" s="25" t="inlineStr">
         <is>
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="K4" s="21" t="inlineStr">
+      <c r="K4" s="25" t="inlineStr">
         <is>
           <t>Spend vs budget %</t>
         </is>
       </c>
-      <c r="L4" s="21" t="inlineStr">
+      <c r="L4" s="25" t="inlineStr">
         <is>
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="M4" s="21" t="inlineStr">
+      <c r="M4" s="25" t="inlineStr">
         <is>
           <t>Months left</t>
         </is>
@@ -1925,7 +3737,7 @@
           <t>State Department of Families</t>
         </is>
       </c>
-      <c r="C5" s="22" t="n">
+      <c r="C5" s="23" t="n">
         <v>480000</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -1938,28 +3750,28 @@
           <t>2027-06-30</t>
         </is>
       </c>
-      <c r="F5" s="22" t="n">
+      <c r="F5" s="23" t="n">
         <v>300000</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="23" t="n">
         <v>306300</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="23" t="n">
         <v>21500</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="23" t="n">
         <v>22800</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="23" t="n">
         <v>300000</v>
       </c>
       <c r="K5" s="8" t="n">
         <v>102.1</v>
       </c>
-      <c r="L5" s="22" t="n">
+      <c r="L5" s="23" t="n">
         <v>173700</v>
       </c>
-      <c r="M5" s="22" t="n">
+      <c r="M5" s="23" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1974,7 +3786,7 @@
           <t>State Housing Program</t>
         </is>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="23" t="n">
         <v>360000</v>
       </c>
       <c r="D6" t="inlineStr">
@@ -1987,28 +3799,28 @@
           <t>2026-12-31</t>
         </is>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="23" t="n">
         <v>360000</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="G6" s="23" t="n">
         <v>257700</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="23" t="n">
         <v>30500</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="23" t="n">
         <v>31200</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="23" t="n">
         <v>270000</v>
       </c>
       <c r="K6" s="8" t="n">
         <v>95.40000000000001</v>
       </c>
-      <c r="L6" s="22" t="n">
+      <c r="L6" s="23" t="n">
         <v>102300</v>
       </c>
-      <c r="M6" s="22" t="n">
+      <c r="M6" s="23" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2023,7 +3835,7 @@
           <t>Local council community grant</t>
         </is>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>48000</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -2036,28 +3848,28 @@
           <t>2027-06-30</t>
         </is>
       </c>
-      <c r="F7" s="22" t="n">
+      <c r="F7" s="23" t="n">
         <v>48000</v>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="G7" s="23" t="n">
         <v>12000</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="23" t="n">
         <v>4100</v>
       </c>
-      <c r="I7" s="22" t="n">
+      <c r="I7" s="23" t="n">
         <v>4300</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="J7" s="23" t="n">
         <v>12000</v>
       </c>
       <c r="K7" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="L7" s="22" t="n">
+      <c r="L7" s="23" t="n">
         <v>36000</v>
       </c>
-      <c r="M7" s="22" t="n">
+      <c r="M7" s="23" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2072,7 +3884,7 @@
           <t>Philanthropic foundation</t>
         </is>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>90000</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -2085,28 +3897,28 @@
           <t>2027-03-31</t>
         </is>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="23" t="n">
         <v>45000</v>
       </c>
-      <c r="G8" s="22" t="n">
+      <c r="G8" s="23" t="n">
         <v>59600</v>
       </c>
-      <c r="H8" s="22" t="n">
+      <c r="H8" s="23" t="n">
         <v>5200</v>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="I8" s="23" t="n">
         <v>4900</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="J8" s="23" t="n">
         <v>60000</v>
       </c>
       <c r="K8" s="8" t="n">
         <v>99.3</v>
       </c>
-      <c r="L8" s="22" t="n">
+      <c r="L8" s="23" t="n">
         <v>30400</v>
       </c>
-      <c r="M8" s="22" t="n">
+      <c r="M8" s="23" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2121,7 +3933,7 @@
           <t>Federal health program</t>
         </is>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>120000</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -2134,28 +3946,28 @@
           <t>2027-03-31</t>
         </is>
       </c>
-      <c r="F9" s="22" t="n">
+      <c r="F9" s="23" t="n">
         <v>60000</v>
       </c>
-      <c r="G9" s="22" t="n">
+      <c r="G9" s="23" t="n">
         <v>57200</v>
       </c>
-      <c r="H9" s="22" t="n">
+      <c r="H9" s="23" t="n">
         <v>9400</v>
       </c>
-      <c r="I9" s="22" t="n">
+      <c r="I9" s="23" t="n">
         <v>10800</v>
       </c>
-      <c r="J9" s="22" t="n">
+      <c r="J9" s="23" t="n">
         <v>60000</v>
       </c>
       <c r="K9" s="8" t="n">
         <v>95.3</v>
       </c>
-      <c r="L9" s="22" t="n">
+      <c r="L9" s="23" t="n">
         <v>62800</v>
       </c>
-      <c r="M9" s="22" t="n">
+      <c r="M9" s="23" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2170,7 +3982,7 @@
           <t>State volunteering grant</t>
         </is>
       </c>
-      <c r="C10" s="22" t="n">
+      <c r="C10" s="23" t="n">
         <v>36000</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -2183,28 +3995,28 @@
           <t>2027-02-28</t>
         </is>
       </c>
-      <c r="F10" s="22" t="n">
+      <c r="F10" s="23" t="n">
         <v>36000</v>
       </c>
-      <c r="G10" s="22" t="n">
+      <c r="G10" s="23" t="n">
         <v>21000</v>
       </c>
-      <c r="H10" s="22" t="n">
+      <c r="H10" s="23" t="n">
         <v>3000</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="I10" s="23" t="n">
         <v>3000</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="23" t="n">
         <v>21000</v>
       </c>
       <c r="K10" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="L10" s="22" t="n">
+      <c r="L10" s="23" t="n">
         <v>15000</v>
       </c>
-      <c r="M10" s="22" t="n">
+      <c r="M10" s="23" t="n">
         <v>5</v>
       </c>
     </row>
@@ -2214,7 +4026,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2249,36 +4061,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>A Brisbane community services charity funded by six grants, donations, events and program fees. About 18 staff. Registered charity, income-tax exempt.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Reporting month</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>September 2026, compared with August 2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Financial year</t>
         </is>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>FY2027: 1 July 2026 to 30 June 2027</t>
         </is>
@@ -2292,96 +4104,96 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Youth outreach</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>State Department of Families: $480,000, 2025-07 to 2027-06</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>Housing support</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>State Housing Program: $360,000, 2026-01 to 2026-12</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>Community meals</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>Local council community grant: $48,000, 2026-07 to 2027-06</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="26" t="inlineStr">
         <is>
           <t>Digital literacy</t>
         </is>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>Philanthropic foundation: $90,000, 2025-10 to 2027-03</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Mental health first aid</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>Federal health program: $120,000, 2026-04 to 2027-03</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Volunteer coordinator</t>
         </is>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>State volunteering grant: $36,000, 2026-03 to 2027-02</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Grant income</t>
         </is>
       </c>
-      <c r="B16" s="24" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>recognised as the money is spent on the program</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Unspent grants</t>
         </is>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>instalments received but not yet spent are a liability (grants received in advance)</t>
         </is>
@@ -2395,48 +4207,48 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Donations</t>
         </is>
       </c>
-      <c r="B20" s="24" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>including the spring appeal in September</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Fundraising event</t>
         </is>
       </c>
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>September gala: income and costs in the same month</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="26" t="inlineStr">
         <is>
           <t>Grant-funded spending</t>
         </is>
       </c>
-      <c r="B22" s="24" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>75% wages, the rest program costs</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="inlineStr">
+      <c r="A23" s="26" t="inlineStr">
         <is>
           <t>Income tax</t>
         </is>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>none: registered charity, income-tax exempt</t>
         </is>
@@ -2450,60 +4262,60 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
+      <c r="A26" s="26" t="inlineStr">
         <is>
           <t>Suppliers</t>
         </is>
       </c>
-      <c r="B26" s="24" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>paid the following month</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="26" t="inlineStr">
         <is>
           <t>Unrestricted cash</t>
         </is>
       </c>
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>cash at bank less unspent grant money</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="23" t="inlineStr">
+      <c r="A28" s="26" t="inlineStr">
         <is>
           <t>Cash runway</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>unrestricted cash ÷ this month's cash spending</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="inlineStr">
+      <c r="A29" s="26" t="inlineStr">
         <is>
           <t>Reserves target</t>
         </is>
       </c>
-      <c r="B29" s="24" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>3 months of spending</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="A30" s="26" t="inlineStr">
         <is>
           <t>GST</t>
         </is>
       </c>
-      <c r="B30" s="24" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>excluded throughout, for simplicity</t>
         </is>

</xml_diff>

<commit_message>
Data status everywhere; professional, printable exports; target line on top
- tools/data_status.py: Locked (closed on the 2nd working day of the
  next month) / Provisional (over, not locked) / Incomplete (today or
  month to date), worked out from the run time. Shown on the dashboard
  (chip, statement headers, assumptions), the deliveries map (per
  period), every export (status panel, footers, Excel header line) and
  in the database (dim_date day_status, month_status, month_locked_on)
- tools/exportkit.py: vector bar charts for PDFs, status panel, page
  X of Y footers, Excel print setup (A4, fit to width, repeated header
  rows, footers, no gridlines)
- Target line drawn on top of the bars; value labels step past it
- Bars sorted by value; negatives in accounting brackets; darker brick
  so late/overdue still separates in black-and-white print

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/nfp-sample-statements.xlsx
+++ b/media/exports/nfp-sample-statements.xlsx
@@ -16,7 +16,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'PandL'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Balance sheet'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Cash flow'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Grants'!$A$4:$M$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Grants'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -541,7 +545,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -566,6 +570,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -647,11 +658,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Community meals</t>
+          <t>Mental health first aid</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>100</v>
+        <v>95.3</v>
       </c>
     </row>
     <row r="12">
@@ -667,11 +678,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mental health first aid</t>
+          <t>Community meals</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>95.3</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -695,7 +706,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -728,6 +749,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1238,8 +1266,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToWidth="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1272,6 +1309,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1537,8 +1581,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToWidth="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1571,6 +1624,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
         <is>
@@ -1812,8 +1872,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" fitToWidth="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1821,7 +1890,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:C172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1845,6 +1914,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -2084,12 +2160,12 @@
       </c>
       <c r="B23" s="22" t="inlineStr">
         <is>
-          <t>$-156,100</t>
+          <t>($156,100)</t>
         </is>
       </c>
       <c r="C23" s="22" t="inlineStr">
         <is>
-          <t>$-221,900</t>
+          <t>($221,900)</t>
         </is>
       </c>
     </row>
@@ -2783,14 +2859,14 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>Community meals</t>
+          <t>Mental health first aid</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>Local council community grant · $48,000 · Jul 2026 to Jun 2027</t>
+          <t>Federal health program · $120,000 · Apr 2026 to Mar 2027</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2886,7 @@
       </c>
       <c r="B94" s="22" t="inlineStr">
         <is>
-          <t>$48,000</t>
+          <t>$60,000</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2898,7 @@
       </c>
       <c r="B95" s="22" t="inlineStr">
         <is>
-          <t>$36,000</t>
+          <t>$62,800</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2910,7 @@
       </c>
       <c r="B96" s="22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2922,7 @@
       </c>
       <c r="B97" s="22" t="inlineStr">
         <is>
-          <t>$12,000</t>
+          <t>$57,200</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2934,7 @@
       </c>
       <c r="B98" s="22" t="inlineStr">
         <is>
-          <t>$12,000</t>
+          <t>$60,000</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2946,7 @@
       </c>
       <c r="B99" s="22" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>95.3%</t>
         </is>
       </c>
     </row>
@@ -2901,207 +2977,207 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Jul 26</t>
+          <t>Apr 26</t>
         </is>
       </c>
       <c r="B103" s="23" t="n">
-        <v>3600</v>
+        <v>9584</v>
       </c>
       <c r="C103" s="23" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Aug 26</t>
+          <t>May 26</t>
         </is>
       </c>
       <c r="B104" s="23" t="n">
-        <v>4100</v>
+        <v>8950</v>
       </c>
       <c r="C104" s="23" t="n">
-        <v>4000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
+          <t>Jun 26</t>
+        </is>
+      </c>
+      <c r="B105" s="23" t="n">
+        <v>9797</v>
+      </c>
+      <c r="C105" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B106" s="23" t="n">
+        <v>8669</v>
+      </c>
+      <c r="C106" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B107" s="23" t="n">
+        <v>9400</v>
+      </c>
+      <c r="C107" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B105" s="23" t="n">
-        <v>4300</v>
-      </c>
-      <c r="C105" s="23" t="n">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="4" t="inlineStr">
+      <c r="B108" s="23" t="n">
+        <v>10800</v>
+      </c>
+      <c r="C108" s="23" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>Digital literacy</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="9" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="9" t="inlineStr">
         <is>
           <t>Philanthropic foundation · $90,000 · Oct 2025 to Mar 2027</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="20" t="inlineStr"/>
-      <c r="B110" s="20" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="20" t="inlineStr"/>
+      <c r="B113" s="20" t="inlineStr">
         <is>
           <t>Sep 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="21" t="inlineStr">
-        <is>
-          <t>Received from the funder</t>
-        </is>
-      </c>
-      <c r="B111" s="22" t="inlineStr">
-        <is>
-          <t>$45,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="21" t="inlineStr">
-        <is>
-          <t>Still to spend</t>
-        </is>
-      </c>
-      <c r="B112" s="22" t="inlineStr">
-        <is>
-          <t>$30,400</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="21" t="inlineStr">
-        <is>
-          <t>Months left</t>
-        </is>
-      </c>
-      <c r="B113" s="22" t="inlineStr">
-        <is>
-          <t>6</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="21" t="inlineStr">
         <is>
-          <t>Spent to date</t>
+          <t>Received from the funder</t>
         </is>
       </c>
       <c r="B114" s="22" t="inlineStr">
         <is>
-          <t>$59,600</t>
+          <t>$45,000</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="21" t="inlineStr">
         <is>
-          <t>Budget to date</t>
+          <t>Still to spend</t>
         </is>
       </c>
       <c r="B115" s="22" t="inlineStr">
         <is>
-          <t>$60,000</t>
+          <t>$30,400</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="21" t="inlineStr">
         <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B116" s="22" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B117" s="22" t="inlineStr">
+        <is>
+          <t>$59,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B118" s="22" t="inlineStr">
+        <is>
+          <t>$60,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="21" t="inlineStr">
+        <is>
           <t>Spent against budget</t>
         </is>
       </c>
-      <c r="B116" s="22" t="inlineStr">
+      <c r="B119" s="22" t="inlineStr">
         <is>
           <t>99.3%</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="7" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="7" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="20" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="20" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B119" s="20" t="inlineStr">
+      <c r="B122" s="20" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="C119" s="20" t="inlineStr">
+      <c r="C122" s="20" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>Oct 25</t>
-        </is>
-      </c>
-      <c r="B120" s="23" t="n">
-        <v>5160</v>
-      </c>
-      <c r="C120" s="23" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t>Nov 25</t>
-        </is>
-      </c>
-      <c r="B121" s="23" t="n">
-        <v>4585</v>
-      </c>
-      <c r="C121" s="23" t="n">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="inlineStr">
-        <is>
-          <t>Dec 25</t>
-        </is>
-      </c>
-      <c r="B122" s="23" t="n">
-        <v>5221</v>
-      </c>
-      <c r="C122" s="23" t="n">
-        <v>5000</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Jan 26</t>
+          <t>Oct 25</t>
         </is>
       </c>
       <c r="B123" s="23" t="n">
-        <v>4426</v>
+        <v>5160</v>
       </c>
       <c r="C123" s="23" t="n">
         <v>5000</v>
@@ -3110,11 +3186,11 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Feb 26</t>
+          <t>Nov 25</t>
         </is>
       </c>
       <c r="B124" s="23" t="n">
-        <v>5408</v>
+        <v>4585</v>
       </c>
       <c r="C124" s="23" t="n">
         <v>5000</v>
@@ -3123,11 +3199,11 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Mar 26</t>
+          <t>Dec 25</t>
         </is>
       </c>
       <c r="B125" s="23" t="n">
-        <v>5427</v>
+        <v>5221</v>
       </c>
       <c r="C125" s="23" t="n">
         <v>5000</v>
@@ -3136,11 +3212,11 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Apr 26</t>
+          <t>Jan 26</t>
         </is>
       </c>
       <c r="B126" s="23" t="n">
-        <v>5509</v>
+        <v>4426</v>
       </c>
       <c r="C126" s="23" t="n">
         <v>5000</v>
@@ -3149,11 +3225,11 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>May 26</t>
+          <t>Feb 26</t>
         </is>
       </c>
       <c r="B127" s="23" t="n">
-        <v>4635</v>
+        <v>5408</v>
       </c>
       <c r="C127" s="23" t="n">
         <v>5000</v>
@@ -3162,11 +3238,11 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Jun 26</t>
+          <t>Mar 26</t>
         </is>
       </c>
       <c r="B128" s="23" t="n">
-        <v>4316</v>
+        <v>5427</v>
       </c>
       <c r="C128" s="23" t="n">
         <v>5000</v>
@@ -3175,11 +3251,11 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Jul 26</t>
+          <t>Apr 26</t>
         </is>
       </c>
       <c r="B129" s="23" t="n">
-        <v>4813</v>
+        <v>5509</v>
       </c>
       <c r="C129" s="23" t="n">
         <v>5000</v>
@@ -3188,11 +3264,11 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Aug 26</t>
+          <t>May 26</t>
         </is>
       </c>
       <c r="B130" s="23" t="n">
-        <v>5200</v>
+        <v>4635</v>
       </c>
       <c r="C130" s="23" t="n">
         <v>5000</v>
@@ -3201,171 +3277,171 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Sep 26</t>
+          <t>Jun 26</t>
         </is>
       </c>
       <c r="B131" s="23" t="n">
-        <v>4900</v>
+        <v>4316</v>
       </c>
       <c r="C131" s="23" t="n">
         <v>5000</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B132" s="23" t="n">
+        <v>4813</v>
+      </c>
+      <c r="C132" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Aug 26</t>
+        </is>
+      </c>
+      <c r="B133" s="23" t="n">
+        <v>5200</v>
+      </c>
+      <c r="C133" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
     <row r="134">
-      <c r="A134" s="4" t="inlineStr">
-        <is>
-          <t>Mental health first aid</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="9" t="inlineStr">
-        <is>
-          <t>Federal health program · $120,000 · Apr 2026 to Mar 2027</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="20" t="inlineStr"/>
-      <c r="B136" s="20" t="inlineStr">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Sep 26</t>
+        </is>
+      </c>
+      <c r="B134" s="23" t="n">
+        <v>4900</v>
+      </c>
+      <c r="C134" s="23" t="n">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>Community meals</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="inlineStr">
+        <is>
+          <t>Local council community grant · $48,000 · Jul 2026 to Jun 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="20" t="inlineStr"/>
+      <c r="B139" s="20" t="inlineStr">
         <is>
           <t>Sep 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="21" t="inlineStr">
-        <is>
-          <t>Received from the funder</t>
-        </is>
-      </c>
-      <c r="B137" s="22" t="inlineStr">
-        <is>
-          <t>$60,000</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="21" t="inlineStr">
-        <is>
-          <t>Still to spend</t>
-        </is>
-      </c>
-      <c r="B138" s="22" t="inlineStr">
-        <is>
-          <t>$62,800</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="21" t="inlineStr">
-        <is>
-          <t>Months left</t>
-        </is>
-      </c>
-      <c r="B139" s="22" t="inlineStr">
-        <is>
-          <t>6</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="21" t="inlineStr">
         <is>
-          <t>Spent to date</t>
+          <t>Received from the funder</t>
         </is>
       </c>
       <c r="B140" s="22" t="inlineStr">
         <is>
-          <t>$57,200</t>
+          <t>$48,000</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="21" t="inlineStr">
         <is>
-          <t>Budget to date</t>
+          <t>Still to spend</t>
         </is>
       </c>
       <c r="B141" s="22" t="inlineStr">
         <is>
-          <t>$60,000</t>
+          <t>$36,000</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="21" t="inlineStr">
         <is>
+          <t>Months left</t>
+        </is>
+      </c>
+      <c r="B142" s="22" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="21" t="inlineStr">
+        <is>
+          <t>Spent to date</t>
+        </is>
+      </c>
+      <c r="B143" s="22" t="inlineStr">
+        <is>
+          <t>$12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="21" t="inlineStr">
+        <is>
+          <t>Budget to date</t>
+        </is>
+      </c>
+      <c r="B144" s="22" t="inlineStr">
+        <is>
+          <t>$12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="21" t="inlineStr">
+        <is>
           <t>Spent against budget</t>
         </is>
       </c>
-      <c r="B142" s="22" t="inlineStr">
-        <is>
-          <t>95.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="7" t="inlineStr">
+      <c r="B145" s="22" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="7" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="20" t="inlineStr">
+    <row r="148">
+      <c r="A148" s="20" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="B145" s="20" t="inlineStr">
+      <c r="B148" s="20" t="inlineStr">
         <is>
           <t>Spend</t>
         </is>
       </c>
-      <c r="C145" s="20" t="inlineStr">
+      <c r="C148" s="20" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Apr 26</t>
-        </is>
-      </c>
-      <c r="B146" s="23" t="n">
-        <v>9584</v>
-      </c>
-      <c r="C146" s="23" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>May 26</t>
-        </is>
-      </c>
-      <c r="B147" s="23" t="n">
-        <v>8950</v>
-      </c>
-      <c r="C147" s="23" t="n">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>Jun 26</t>
-        </is>
-      </c>
-      <c r="B148" s="23" t="n">
-        <v>9797</v>
-      </c>
-      <c r="C148" s="23" t="n">
-        <v>10000</v>
       </c>
     </row>
     <row r="149">
@@ -3375,10 +3451,10 @@
         </is>
       </c>
       <c r="B149" s="23" t="n">
-        <v>8669</v>
+        <v>3600</v>
       </c>
       <c r="C149" s="23" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="150">
@@ -3388,10 +3464,10 @@
         </is>
       </c>
       <c r="B150" s="23" t="n">
-        <v>9400</v>
+        <v>4100</v>
       </c>
       <c r="C150" s="23" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="151">
@@ -3401,10 +3477,10 @@
         </is>
       </c>
       <c r="B151" s="23" t="n">
-        <v>10800</v>
+        <v>4300</v>
       </c>
       <c r="C151" s="23" t="n">
-        <v>10000</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="154">
@@ -3617,7 +3693,17 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -3625,7 +3711,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -3659,6 +3745,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="24" t="inlineStr">
         <is>
@@ -4022,7 +4115,17 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:M10"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -4030,7 +4133,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -4053,6 +4156,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (as at 2pm, Tue 6 Oct 2026)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -4371,6 +4481,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.7" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 Printed 6 Oct 2026</oddHeader>
+    <oddFooter>&amp;L&amp;8 The 4th Sheet · Sample data&amp;C&amp;8 Sep 2026 locked · Oct 2026 incomplete · as at 2pm, Tue 6 Oct 2026&amp;R&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Review phase 6: downloads rebuilt; trades and services never mixed; generated stamps and full download names; made-with notes
Excel: native charts, tables, named headline numbers, points and direction colours, Roboto on every cell.
PowerPoint: real layouts and theme, one slide per topic, target and break-even lines, speaker notes.
PDF: dollar shortfall instead of ticks, tables flow, no forced page gaps.
Separation: per-business growth downloads, business named in every working, Power BI one-business guards,
tools/tests/org_separation.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/nfp-sample-statements.xlsx
+++ b/media/exports/nfp-sample-statements.xlsx
@@ -16,12 +16,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="Cost_to_raise_a_dollar">'The fourth sheet'!$B$6</definedName>
+    <definedName name="Unrestricted_cash_runway">'The fourth sheet'!$B$7</definedName>
+    <definedName name="Grants_ending_in_6_months">'The fourth sheet'!$B$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'The fourth sheet'!$5:$5</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'The fourth sheet'!$A$1:$D$19</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Income and expenditure'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Income and expenditure'!$A$1:$D$35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Balance sheet'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Balance sheet'!$A$1:$D$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Cash flow'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Grants'!$A$6:$M$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Cash flow'!$A$1:$D$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Grants'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Grants'!$A$1:$M$13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'Workings'!$A$1:$D$191</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Assumptions'!$A$1:$B$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -29,13 +38,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="#,##0;[Red](#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0&quot;¢&quot;;[Red](0&quot;¢&quot;)"/>
     <numFmt numFmtId="166" formatCode="0.0&quot; months&quot;;[Red](0.0&quot; months&quot;)"/>
     <numFmt numFmtId="167" formatCode="0.0%;[Red](0.0%);&quot;-&quot;"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="169" formatCode="d mmm yyyy"/>
+    <numFmt numFmtId="168" formatCode="+0&quot;¢&quot;;(0&quot;¢&quot;);&quot;-&quot;"/>
+    <numFmt numFmtId="169" formatCode="+0.0&quot; months&quot;;(0.0&quot; months&quot;);&quot;-&quot;"/>
+    <numFmt numFmtId="170" formatCode="+#,##0;(#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="172" formatCode="d mmm yyyy"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -148,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,7 +171,9 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -167,18 +181,18 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment indent="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="12" fillId="3" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -213,6 +227,22 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <name val="Roboto"/>
+        <b val="1"/>
+        <color rgb="00B42318"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Roboto"/>
+        <b val="1"/>
+        <color rgb="002F7A5D"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -283,6 +313,338 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="25342A"/>
+                </a:solidFill>
+                <a:latin typeface="Roboto"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="25342A"/>
+                </a:solidFill>
+                <a:latin typeface="Roboto"/>
+              </a:rPr>
+              <a:t>Each grant: over or under budget to 30 September 2026</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <varyColors val="0"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>% of budget</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0E9F6E"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="0E9F6E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <invertIfNegative val="0"/>
+          <dPt>
+            <idx val="0"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="B42318"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="1"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="B42318"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dPt>
+            <idx val="2"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="B42318"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="B42318"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </dPt>
+          <dLbls>
+            <numFmt formatCode="0.0%"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'The fourth sheet'!$A$14:$A$19</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'The fourth sheet'!$B$14:$B$19</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <numFmt formatCode="0.0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="25342A"/>
+                </a:solidFill>
+                <a:latin typeface="Roboto"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr sz="1100" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="25342A"/>
+                </a:solidFill>
+                <a:latin typeface="Roboto"/>
+              </a:rPr>
+              <a:t>Spent against budget to date</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+      <overlay val="0"/>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <varyColors val="0"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Spent against budget to date</v>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="0E9F6E"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
+                <a:srgbClr val="0E9F6E"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <invertIfNegative val="0"/>
+          <dLbls>
+            <numFmt formatCode="0.0%"/>
+            <showLegendKey val="0"/>
+            <showVal val="1"/>
+            <showCatName val="0"/>
+            <showSerName val="0"/>
+            <showPercent val="0"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'Grants'!$A$7:$A$12</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Grants'!$K$7:$K$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="60"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="maxMin"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <delete val="1"/>
+        <axPos val="l"/>
+        <numFmt formatCode="0.0%" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>11</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2340000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>14</col>
+      <colOff>0</colOff>
+      <row>5</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2340000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Grants" displayName="Grants" ref="A6:M12" headerRowCount="1">
+  <autoFilter ref="A6:M12"/>
+  <tableColumns count="13">
+    <tableColumn id="1" name="Program"/>
+    <tableColumn id="2" name="Funder"/>
+    <tableColumn id="3" name="Grant total"/>
+    <tableColumn id="4" name="Start"/>
+    <tableColumn id="5" name="End"/>
+    <tableColumn id="6" name="Received to date"/>
+    <tableColumn id="7" name="Spent to date"/>
+    <tableColumn id="8" name="Spent Aug"/>
+    <tableColumn id="9" name="Spent Sep"/>
+    <tableColumn id="10" name="Budget to date"/>
+    <tableColumn id="11" name="Spent against budget"/>
+    <tableColumn id="12" name="Still to spend"/>
+    <tableColumn id="13" name="Months left"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -593,14 +955,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
@@ -641,7 +1003,7 @@
         <f>Workings!C16</f>
         <v/>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="6">
         <f>B6-C6</f>
         <v/>
       </c>
@@ -652,15 +1014,15 @@
           <t>Unrestricted cash runway</t>
         </is>
       </c>
-      <c r="B7" s="6">
+      <c r="B7" s="7">
         <f>Workings!B27</f>
         <v/>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="7">
         <f>Workings!C27</f>
         <v/>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="8">
         <f>B7-C7</f>
         <v/>
       </c>
@@ -671,7 +1033,7 @@
           <t>Grants ending in 6 months</t>
         </is>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="9">
         <f>Workings!B36</f>
         <v/>
       </c>
@@ -679,7 +1041,7 @@
     <row r="9"/>
     <row r="10"/>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Each grant: over or under budget to 30 September 2026</t>
         </is>
@@ -711,11 +1073,11 @@
           <t>Youth outreach</t>
         </is>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="11">
         <f>Workings!B50</f>
         <v/>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="9">
         <f>Workings!B49</f>
         <v/>
       </c>
@@ -726,11 +1088,11 @@
           <t>Housing support</t>
         </is>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="11">
         <f>Workings!B82</f>
         <v/>
       </c>
-      <c r="C15" s="7">
+      <c r="C15" s="9">
         <f>Workings!B81</f>
         <v/>
       </c>
@@ -741,11 +1103,11 @@
           <t>Mental health first aid</t>
         </is>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="11">
         <f>Workings!B108</f>
         <v/>
       </c>
-      <c r="C16" s="7">
+      <c r="C16" s="9">
         <f>Workings!B107</f>
         <v/>
       </c>
@@ -756,11 +1118,11 @@
           <t>Digital literacy</t>
         </is>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="11">
         <f>Workings!B131</f>
         <v/>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="9">
         <f>Workings!B130</f>
         <v/>
       </c>
@@ -771,11 +1133,11 @@
           <t>Community meals</t>
         </is>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="11">
         <f>Workings!B160</f>
         <v/>
       </c>
-      <c r="C18" s="7">
+      <c r="C18" s="9">
         <f>Workings!B159</f>
         <v/>
       </c>
@@ -786,27 +1148,44 @@
           <t>Volunteer coordinator</t>
         </is>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="11">
         <f>Workings!B180</f>
         <v/>
       </c>
-      <c r="C19" s="7">
+      <c r="C19" s="9">
         <f>Workings!B179</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D6">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -835,14 +1214,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
@@ -869,511 +1248,727 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Youth outreach grant</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="9" t="n">
         <v>22800</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="9" t="n">
         <v>21500</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="14">
         <f>B6-C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Housing support grant</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="9" t="n">
         <v>31200</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="9" t="n">
         <v>30500</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="14">
         <f>B7-C7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Community meals grant</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="9" t="n">
         <v>4300</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="9" t="n">
         <v>4100</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="14">
         <f>B8-C8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Digital literacy grant</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="9" t="n">
         <v>4900</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="9" t="n">
         <v>5200</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="14">
         <f>B9-C9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Mental health first aid grant</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="9" t="n">
         <v>10800</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="9" t="n">
         <v>9400</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="14">
         <f>B10-C10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Volunteer coordinator grant</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="14">
         <f>B11-C11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Donations</t>
         </is>
       </c>
-      <c r="B12" s="7" t="n">
+      <c r="B12" s="9" t="n">
         <v>27900</v>
       </c>
-      <c r="C12" s="7" t="n">
+      <c r="C12" s="9" t="n">
         <v>18400</v>
       </c>
-      <c r="D12" s="12">
+      <c r="D12" s="14">
         <f>B12-C12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Fundraising events</t>
         </is>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="9" t="n">
         <v>41600</v>
       </c>
-      <c r="C13" s="7" t="n">
+      <c r="C13" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="12">
+      <c r="D13" s="14">
         <f>B13-C13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Program fees</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="9" t="n">
         <v>28300</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="9" t="n">
         <v>26800</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="14">
         <f>B14-C14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Interest</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <v>1380</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="9" t="n">
         <v>1450</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="14">
         <f>B15-C15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Total income</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="16">
         <f>SUM(B6:B15)</f>
         <v/>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="16">
         <f>SUM(C6:C15)</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="17">
         <f>B16-C16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Programs</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Grant-funded program wages</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n">
+      <c r="B18" s="9" t="n">
         <v>-57750</v>
       </c>
-      <c r="C18" s="7" t="n">
+      <c r="C18" s="9" t="n">
         <v>-55275</v>
       </c>
-      <c r="D18" s="12">
+      <c r="D18" s="14">
         <f>B18-C18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Grant-funded program costs</t>
         </is>
       </c>
-      <c r="B19" s="7" t="n">
+      <c r="B19" s="9" t="n">
         <v>-19250</v>
       </c>
-      <c r="C19" s="7" t="n">
+      <c r="C19" s="9" t="n">
         <v>-18425</v>
       </c>
-      <c r="D19" s="12">
+      <c r="D19" s="14">
         <f>B19-C19</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>Program delivery wages (untied)</t>
         </is>
       </c>
-      <c r="B20" s="7" t="n">
+      <c r="B20" s="9" t="n">
         <v>-14500</v>
       </c>
-      <c r="C20" s="7" t="n">
+      <c r="C20" s="9" t="n">
         <v>-14000</v>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="14">
         <f>B20-C20</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Program costs (untied)</t>
         </is>
       </c>
-      <c r="B21" s="7" t="n">
+      <c r="B21" s="9" t="n">
         <v>-6100</v>
       </c>
-      <c r="C21" s="7" t="n">
+      <c r="C21" s="9" t="n">
         <v>-5500</v>
       </c>
-      <c r="D21" s="12">
+      <c r="D21" s="14">
         <f>B21-C21</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Total program spend</t>
         </is>
       </c>
-      <c r="B22" s="14">
+      <c r="B22" s="16">
         <f>SUM(B18:B21)</f>
         <v/>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="16">
         <f>SUM(C18:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="15">
+      <c r="D22" s="17">
         <f>B22-C22</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Fundraising</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Grant writing and reporting</t>
         </is>
       </c>
-      <c r="B24" s="7" t="n">
+      <c r="B24" s="9" t="n">
         <v>-7100</v>
       </c>
-      <c r="C24" s="7" t="n">
+      <c r="C24" s="9" t="n">
         <v>-7100</v>
       </c>
-      <c r="D24" s="12">
+      <c r="D24" s="14">
         <f>B24-C24</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Donor campaigns</t>
         </is>
       </c>
-      <c r="B25" s="7" t="n">
+      <c r="B25" s="9" t="n">
         <v>-5400</v>
       </c>
-      <c r="C25" s="7" t="n">
+      <c r="C25" s="9" t="n">
         <v>-2200</v>
       </c>
-      <c r="D25" s="12">
+      <c r="D25" s="14">
         <f>B25-C25</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>Event costs</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n">
+      <c r="B26" s="9" t="n">
         <v>-16900</v>
       </c>
-      <c r="C26" s="7" t="n">
+      <c r="C26" s="9" t="n">
         <v>-2400</v>
       </c>
-      <c r="D26" s="12">
+      <c r="D26" s="14">
         <f>B26-C26</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Total fundraising costs</t>
         </is>
       </c>
-      <c r="B27" s="14">
+      <c r="B27" s="16">
         <f>SUM(B24:B26)</f>
         <v/>
       </c>
-      <c r="C27" s="14">
+      <c r="C27" s="16">
         <f>SUM(C24:C26)</f>
         <v/>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="17">
         <f>B27-C27</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Administration</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Administration wages</t>
         </is>
       </c>
-      <c r="B29" s="7" t="n">
+      <c r="B29" s="9" t="n">
         <v>-18300</v>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C29" s="9" t="n">
         <v>-18300</v>
       </c>
-      <c r="D29" s="12">
+      <c r="D29" s="14">
         <f>B29-C29</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Occupancy</t>
         </is>
       </c>
-      <c r="B30" s="7" t="n">
+      <c r="B30" s="9" t="n">
         <v>-10000</v>
       </c>
-      <c r="C30" s="7" t="n">
+      <c r="C30" s="9" t="n">
         <v>-10000</v>
       </c>
-      <c r="D30" s="12">
+      <c r="D30" s="14">
         <f>B30-C30</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Other administration</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n">
+      <c r="B31" s="9" t="n">
         <v>-7600</v>
       </c>
-      <c r="C31" s="7" t="n">
+      <c r="C31" s="9" t="n">
         <v>-8000</v>
       </c>
-      <c r="D31" s="12">
+      <c r="D31" s="14">
         <f>B31-C31</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Total administration</t>
         </is>
       </c>
-      <c r="B32" s="14">
+      <c r="B32" s="16">
         <f>SUM(B29:B31)</f>
         <v/>
       </c>
-      <c r="C32" s="14">
+      <c r="C32" s="16">
         <f>SUM(C29:C31)</f>
         <v/>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="17">
         <f>B32-C32</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n">
+      <c r="B33" s="16" t="n">
         <v>-2900</v>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="16" t="n">
         <v>-2900</v>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="17">
         <f>B33-C33</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Total expenses</t>
         </is>
       </c>
-      <c r="B34" s="14">
+      <c r="B34" s="16">
         <f>B22+B27+B32+B33</f>
         <v/>
       </c>
-      <c r="C34" s="14">
+      <c r="C34" s="16">
         <f>C22+C27+C32+C33</f>
         <v/>
       </c>
-      <c r="D34" s="15">
+      <c r="D34" s="17">
         <f>B34-C34</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>Surplus for the month</t>
         </is>
       </c>
-      <c r="B35" s="17">
+      <c r="B35" s="19">
         <f>B16+B34</f>
         <v/>
       </c>
-      <c r="C35" s="17">
+      <c r="C35" s="19">
         <f>C16+C34</f>
         <v/>
       </c>
-      <c r="D35" s="18">
+      <c r="D35" s="20">
         <f>B35-C35</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D6">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D8">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10">
+    <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11">
+    <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
+    <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D13">
+    <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D14">
+    <cfRule type="cellIs" priority="17" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15">
+    <cfRule type="cellIs" priority="19" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="20" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="22" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18">
+    <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="24" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D19">
+    <cfRule type="cellIs" priority="25" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="26" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20">
+    <cfRule type="cellIs" priority="27" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="28" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D21">
+    <cfRule type="cellIs" priority="29" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="30" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22">
+    <cfRule type="cellIs" priority="31" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="32" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D24">
+    <cfRule type="cellIs" priority="33" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="34" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25">
+    <cfRule type="cellIs" priority="35" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="36" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D26">
+    <cfRule type="cellIs" priority="37" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="38" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D27">
+    <cfRule type="cellIs" priority="39" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="40" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D29">
+    <cfRule type="cellIs" priority="41" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="42" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D30">
+    <cfRule type="cellIs" priority="43" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="44" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D31">
+    <cfRule type="cellIs" priority="45" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="46" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D32">
+    <cfRule type="cellIs" priority="47" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="48" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D33">
+    <cfRule type="cellIs" priority="49" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="50" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D34">
+    <cfRule type="cellIs" priority="51" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="52" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D35">
+    <cfRule type="cellIs" priority="53" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="54" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1410,14 +2005,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
@@ -1444,251 +2039,251 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Current assets</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Cash at bank</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="9" t="n">
         <v>480780</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="9" t="n">
         <v>525675</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="14">
         <f>B6-C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Program fees receivable</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="9" t="n">
         <v>10400</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="9" t="n">
         <v>9800</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="14">
         <f>B7-C7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Grants receivable (spent ahead of instalment)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="9" t="n">
         <v>20900</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="9" t="n">
         <v>9700</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="14">
         <f>B8-C8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Prepayments</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="9" t="n">
         <v>21000</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="9" t="n">
         <v>21000</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="14">
         <f>B9-C9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Total current assets</t>
         </is>
       </c>
-      <c r="B10" s="14">
+      <c r="B10" s="16">
         <f>SUM(B6:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="16">
         <f>SUM(C6:C9)</f>
         <v/>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="17">
         <f>B10-C10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Vehicles and equipment</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="16" t="n">
         <v>172200</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="16" t="n">
         <v>175100</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="17">
         <f>B11-C11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="16">
         <f>B10+B11</f>
         <v/>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="16">
         <f>C10+C11</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="17">
         <f>B12-C12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Current liabilities</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Payables (bills due next month)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="9" t="n">
         <v>65250</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="9" t="n">
         <v>46525</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="14">
         <f>B14-C14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>Grants received in advance (unspent)</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <v>156100</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="C15" s="9" t="n">
         <v>221900</v>
       </c>
-      <c r="D15" s="12">
+      <c r="D15" s="14">
         <f>B15-C15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Employee leave provisions</t>
         </is>
       </c>
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="9" t="n">
         <v>166600</v>
       </c>
-      <c r="C16" s="7" t="n">
+      <c r="C16" s="9" t="n">
         <v>165900</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="14">
         <f>B16-C16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="B17" s="14">
+      <c r="B17" s="16">
         <f>SUM(B14:B16)</f>
         <v/>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="16">
         <f>SUM(C14:C16)</f>
         <v/>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="17">
         <f>B17-C17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Net assets</t>
         </is>
       </c>
-      <c r="B18" s="17">
+      <c r="B18" s="19">
         <f>B12-B17</f>
         <v/>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="19">
         <f>C12-C17</f>
         <v/>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="20">
         <f>B18-C18</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Equity</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Accumulated funds</t>
         </is>
       </c>
-      <c r="B20" s="17" t="n">
+      <c r="B20" s="19" t="n">
         <v>317330</v>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="19" t="n">
         <v>306950</v>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="20">
         <f>B20-C20</f>
         <v/>
       </c>
@@ -1699,7 +2294,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1733,14 +2328,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
@@ -1767,238 +2362,334 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Operating activities</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>Grant instalments received</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n">
+      <c r="B6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="C6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="12">
+      <c r="D6" s="14">
         <f>B6-C6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Donations and fundraising received</t>
         </is>
       </c>
-      <c r="B7" s="7" t="n">
+      <c r="B7" s="9" t="n">
         <v>69500</v>
       </c>
-      <c r="C7" s="7" t="n">
+      <c r="C7" s="9" t="n">
         <v>18400</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="14">
         <f>B7-C7</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Program fees received</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B8" s="9" t="n">
         <v>27700</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="9" t="n">
         <v>26100</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="14">
         <f>B8-C8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Interest received</t>
         </is>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="9" t="n">
         <v>1380</v>
       </c>
-      <c r="C9" s="7" t="n">
+      <c r="C9" s="9" t="n">
         <v>1450</v>
       </c>
-      <c r="D9" s="12">
+      <c r="D9" s="14">
         <f>B9-C9</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Payments to suppliers</t>
         </is>
       </c>
-      <c r="B10" s="7" t="n">
+      <c r="B10" s="9" t="n">
         <v>-46525</v>
       </c>
-      <c r="C10" s="7" t="n">
+      <c r="C10" s="9" t="n">
         <v>-36500</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="14">
         <f>B10-C10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>Payments to employees</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="9" t="n">
         <v>-96950</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="9" t="n">
         <v>-93775</v>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="14">
         <f>B11-C11</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Net cash from operating activities</t>
         </is>
       </c>
-      <c r="B12" s="14">
+      <c r="B12" s="16">
         <f>SUM(B6:B11)</f>
         <v/>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="16">
         <f>SUM(C6:C11)</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="17">
         <f>B12-C12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Investing activities</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Purchase of vehicles and equipment</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
+      <c r="B14" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="C14" s="7" t="n">
+      <c r="C14" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="12">
+      <c r="D14" s="14">
         <f>B14-C14</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Net cash from investing activities</t>
         </is>
       </c>
-      <c r="B15" s="14">
+      <c r="B15" s="16">
         <f>SUM(B14:B14)</f>
         <v/>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="16">
         <f>SUM(C14:C14)</f>
         <v/>
       </c>
-      <c r="D15" s="15">
+      <c r="D15" s="17">
         <f>B15-C15</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="B16" s="14">
+      <c r="B16" s="16">
         <f>B12+B15</f>
         <v/>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="16">
         <f>C12+C15</f>
         <v/>
       </c>
-      <c r="D16" s="15">
+      <c r="D16" s="17">
         <f>B16-C16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Cash at start of month</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="16" t="n">
         <v>525675</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="16" t="n">
         <v>610000</v>
       </c>
-      <c r="D17" s="15">
+      <c r="D17" s="17">
         <f>B17-C17</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Cash at end of month</t>
         </is>
       </c>
-      <c r="B18" s="17">
+      <c r="B18" s="19">
         <f>B17+B16</f>
         <v/>
       </c>
-      <c r="C18" s="17">
+      <c r="C18" s="19">
         <f>C17+C16</f>
         <v/>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="20">
         <f>B18-C18</f>
         <v/>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="D6">
+    <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7">
+    <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D8">
+    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10">
+    <cfRule type="cellIs" priority="9" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11">
+    <cfRule type="cellIs" priority="11" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="12" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
+    <cfRule type="cellIs" priority="13" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="14" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D14">
+    <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="16" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15">
+    <cfRule type="cellIs" priority="17" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="18" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16">
+    <cfRule type="cellIs" priority="19" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="20" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17">
+    <cfRule type="cellIs" priority="21" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="22" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18">
+    <cfRule type="cellIs" priority="23" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="24" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2041,14 +2732,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
@@ -2128,335 +2819,338 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Youth outreach</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>State Department of Families</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="22" t="n">
         <v>480000</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="23" t="n">
         <v>45839</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="23" t="n">
         <v>46568</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="22" t="n">
         <v>300000</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="22" t="n">
         <v>306300</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="22" t="n">
         <v>21500</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="22" t="n">
         <v>22800</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="22" t="n">
         <v>300000</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="24">
         <f>IF(J7=0,"",G7/J7)</f>
         <v/>
       </c>
-      <c r="L7" s="20">
+      <c r="L7" s="22">
         <f>C7-G7</f>
         <v/>
       </c>
-      <c r="M7" s="20" t="n">
+      <c r="M7" s="22" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Housing support</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>State Housing Program</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="22" t="n">
         <v>360000</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="23" t="n">
         <v>46023</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="23" t="n">
         <v>46387</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="22" t="n">
         <v>360000</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="22" t="n">
         <v>257700</v>
       </c>
-      <c r="H8" s="20" t="n">
+      <c r="H8" s="22" t="n">
         <v>30500</v>
       </c>
-      <c r="I8" s="20" t="n">
+      <c r="I8" s="22" t="n">
         <v>31200</v>
       </c>
-      <c r="J8" s="20" t="n">
+      <c r="J8" s="22" t="n">
         <v>270000</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="24">
         <f>IF(J8=0,"",G8/J8)</f>
         <v/>
       </c>
-      <c r="L8" s="20">
+      <c r="L8" s="22">
         <f>C8-G8</f>
         <v/>
       </c>
-      <c r="M8" s="20" t="n">
+      <c r="M8" s="22" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Mental health first aid</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>Federal health program</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="22" t="n">
         <v>120000</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="23" t="n">
         <v>46113</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="23" t="n">
         <v>46477</v>
       </c>
-      <c r="F9" s="20" t="n">
+      <c r="F9" s="22" t="n">
         <v>60000</v>
       </c>
-      <c r="G9" s="20" t="n">
+      <c r="G9" s="22" t="n">
         <v>57200</v>
       </c>
-      <c r="H9" s="20" t="n">
+      <c r="H9" s="22" t="n">
         <v>9400</v>
       </c>
-      <c r="I9" s="20" t="n">
+      <c r="I9" s="22" t="n">
         <v>10800</v>
       </c>
-      <c r="J9" s="20" t="n">
+      <c r="J9" s="22" t="n">
         <v>60000</v>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="24">
         <f>IF(J9=0,"",G9/J9)</f>
         <v/>
       </c>
-      <c r="L9" s="20">
+      <c r="L9" s="22">
         <f>C9-G9</f>
         <v/>
       </c>
-      <c r="M9" s="20" t="n">
+      <c r="M9" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Digital literacy</t>
         </is>
       </c>
-      <c r="B10" s="19" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Philanthropic foundation</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="22" t="n">
         <v>90000</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="23" t="n">
         <v>45931</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="23" t="n">
         <v>46477</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="22" t="n">
         <v>45000</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="22" t="n">
         <v>59600</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="22" t="n">
         <v>5200</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="22" t="n">
         <v>4900</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J10" s="22" t="n">
         <v>60000</v>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="24">
         <f>IF(J10=0,"",G10/J10)</f>
         <v/>
       </c>
-      <c r="L10" s="20">
+      <c r="L10" s="22">
         <f>C10-G10</f>
         <v/>
       </c>
-      <c r="M10" s="20" t="n">
+      <c r="M10" s="22" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Community meals</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Local council community grant</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="22" t="n">
         <v>48000</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="23" t="n">
         <v>46204</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="23" t="n">
         <v>46568</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="22" t="n">
         <v>48000</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="22" t="n">
         <v>12000</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="22" t="n">
         <v>4100</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="22" t="n">
         <v>4300</v>
       </c>
-      <c r="J11" s="20" t="n">
+      <c r="J11" s="22" t="n">
         <v>12000</v>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="24">
         <f>IF(J11=0,"",G11/J11)</f>
         <v/>
       </c>
-      <c r="L11" s="20">
+      <c r="L11" s="22">
         <f>C11-G11</f>
         <v/>
       </c>
-      <c r="M11" s="20" t="n">
+      <c r="M11" s="22" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Volunteer coordinator</t>
         </is>
       </c>
-      <c r="B12" s="19" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>State volunteering grant</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <v>36000</v>
       </c>
-      <c r="D12" s="21" t="n">
+      <c r="D12" s="23" t="n">
         <v>46082</v>
       </c>
-      <c r="E12" s="21" t="n">
+      <c r="E12" s="23" t="n">
         <v>46446</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="22" t="n">
         <v>36000</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="22" t="n">
         <v>21000</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="H12" s="22" t="n">
         <v>3000</v>
       </c>
-      <c r="I12" s="20" t="n">
+      <c r="I12" s="22" t="n">
         <v>3000</v>
       </c>
-      <c r="J12" s="20" t="n">
+      <c r="J12" s="22" t="n">
         <v>21000</v>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="24">
         <f>IF(J12=0,"",G12/J12)</f>
         <v/>
       </c>
-      <c r="L12" s="20">
+      <c r="L12" s="22">
         <f>C12-G12</f>
         <v/>
       </c>
-      <c r="M12" s="20" t="n">
+      <c r="M12" s="22" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C13" s="24">
+      <c r="C13" s="26">
         <f>SUM(C7:C12)</f>
         <v/>
       </c>
-      <c r="F13" s="24">
+      <c r="F13" s="26">
         <f>SUM(F7:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="26">
         <f>SUM(G7:G12)</f>
         <v/>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="26">
         <f>SUM(H7:H12)</f>
         <v/>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="26">
         <f>SUM(I7:I12)</f>
         <v/>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="26">
         <f>SUM(J7:J12)</f>
         <v/>
       </c>
-      <c r="L13" s="24">
+      <c r="L13" s="26">
         <f>SUM(L7:L12)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:M12"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -2485,27 +3179,27 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Cost to raise a dollar</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Fundraising costs ÷ money raised (grants, donations, events), in cents</t>
         </is>
@@ -2530,10 +3224,10 @@
           <t>Grant writing and reporting</t>
         </is>
       </c>
-      <c r="B8" s="20" t="n">
+      <c r="B8" s="22" t="n">
         <v>7100</v>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="22" t="n">
         <v>7100</v>
       </c>
     </row>
@@ -2543,10 +3237,10 @@
           <t>Donor campaigns</t>
         </is>
       </c>
-      <c r="B9" s="20" t="n">
+      <c r="B9" s="22" t="n">
         <v>5400</v>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="22" t="n">
         <v>2200</v>
       </c>
     </row>
@@ -2556,10 +3250,10 @@
           <t>Event costs</t>
         </is>
       </c>
-      <c r="B10" s="20" t="n">
+      <c r="B10" s="22" t="n">
         <v>16900</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="22" t="n">
         <v>2400</v>
       </c>
     </row>
@@ -2569,11 +3263,11 @@
           <t>Fundraising costs</t>
         </is>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="22">
         <f>B8+B9+B10</f>
         <v/>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="22">
         <f>C8+C9+C10</f>
         <v/>
       </c>
@@ -2584,10 +3278,10 @@
           <t>Grant income</t>
         </is>
       </c>
-      <c r="B12" s="20" t="n">
+      <c r="B12" s="22" t="n">
         <v>77000</v>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="22" t="n">
         <v>73700</v>
       </c>
     </row>
@@ -2597,10 +3291,10 @@
           <t>Donations</t>
         </is>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B13" s="22" t="n">
         <v>27900</v>
       </c>
-      <c r="C13" s="20" t="n">
+      <c r="C13" s="22" t="n">
         <v>18400</v>
       </c>
     </row>
@@ -2610,10 +3304,10 @@
           <t>Fundraising events</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n">
+      <c r="B14" s="22" t="n">
         <v>41600</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2623,26 +3317,26 @@
           <t>Money raised</t>
         </is>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="22">
         <f>B12+B13+B14</f>
         <v/>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="22">
         <f>C12+C13+C14</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Cost per dollar raised</t>
         </is>
       </c>
-      <c r="B16" s="28">
+      <c r="B16" s="30">
         <f>B11/B15*100</f>
         <v/>
       </c>
-      <c r="C16" s="28">
+      <c r="C16" s="30">
         <f>C11/C15*100</f>
         <v/>
       </c>
@@ -2657,14 +3351,14 @@
     <row r="18"/>
     <row r="19"/>
     <row r="20">
-      <c r="A20" s="25" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>Unrestricted cash runway</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="26" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>(Cash at bank − unspent grant money) ÷ this month's cash spending</t>
         </is>
@@ -2689,10 +3383,10 @@
           <t>Cash at bank</t>
         </is>
       </c>
-      <c r="B23" s="20" t="n">
+      <c r="B23" s="22" t="n">
         <v>480780</v>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="22" t="n">
         <v>525675</v>
       </c>
     </row>
@@ -2702,10 +3396,10 @@
           <t>Less unspent grant money (belongs to funders' programs)</t>
         </is>
       </c>
-      <c r="B24" s="20" t="n">
+      <c r="B24" s="22" t="n">
         <v>-156100</v>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="22" t="n">
         <v>-221900</v>
       </c>
     </row>
@@ -2715,11 +3409,11 @@
           <t>Unrestricted cash</t>
         </is>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="22">
         <f>B23+B24</f>
         <v/>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="22">
         <f>C23+C24</f>
         <v/>
       </c>
@@ -2730,24 +3424,24 @@
           <t>Cash spending in the month (expenses less depreciation)</t>
         </is>
       </c>
-      <c r="B26" s="20" t="n">
+      <c r="B26" s="22" t="n">
         <v>162900</v>
       </c>
-      <c r="C26" s="20" t="n">
+      <c r="C26" s="22" t="n">
         <v>141200</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Runway</t>
         </is>
       </c>
-      <c r="B27" s="29">
+      <c r="B27" s="31">
         <f>B25/B26</f>
         <v/>
       </c>
-      <c r="C27" s="29">
+      <c r="C27" s="31">
         <f>C25/C26</f>
         <v/>
       </c>
@@ -2762,14 +3456,14 @@
     <row r="29"/>
     <row r="30"/>
     <row r="31">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="27" t="inlineStr">
         <is>
           <t>Grants ending in the next 6 months</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="26" t="inlineStr">
+      <c r="A32" s="28" t="inlineStr">
         <is>
           <t>Grant total − spent to date, for each grant ending soon</t>
         </is>
@@ -2789,7 +3483,7 @@
           <t>Housing support (ends 31 Dec 2026)</t>
         </is>
       </c>
-      <c r="B34" s="20" t="n">
+      <c r="B34" s="22" t="n">
         <v>102300</v>
       </c>
     </row>
@@ -2799,17 +3493,17 @@
           <t>Volunteer coordinator (ends 28 Feb 2027)</t>
         </is>
       </c>
-      <c r="B35" s="20" t="n">
+      <c r="B35" s="22" t="n">
         <v>15000</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="inlineStr">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>Total still to spend</t>
         </is>
       </c>
-      <c r="B36" s="30">
+      <c r="B36" s="32">
         <f>B34+B35</f>
         <v/>
       </c>
@@ -2824,14 +3518,14 @@
     <row r="38"/>
     <row r="39"/>
     <row r="40">
-      <c r="A40" s="25" t="inlineStr">
+      <c r="A40" s="27" t="inlineStr">
         <is>
           <t>Youth outreach</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="26" t="inlineStr">
+      <c r="A41" s="28" t="inlineStr">
         <is>
           <t>State Department of Families · $480,000 · Jul 2025 to Jun 2027</t>
         </is>
@@ -2851,7 +3545,7 @@
           <t>Grant total</t>
         </is>
       </c>
-      <c r="B43" s="20" t="n">
+      <c r="B43" s="22" t="n">
         <v>480000</v>
       </c>
     </row>
@@ -2861,7 +3555,7 @@
           <t>Received from the funder</t>
         </is>
       </c>
-      <c r="B44" s="20" t="n">
+      <c r="B44" s="22" t="n">
         <v>300000</v>
       </c>
     </row>
@@ -2871,7 +3565,7 @@
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="B45" s="20" t="n">
+      <c r="B45" s="22" t="n">
         <v>306300</v>
       </c>
     </row>
@@ -2881,7 +3575,7 @@
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="B46" s="20" t="n">
+      <c r="B46" s="22" t="n">
         <v>300000</v>
       </c>
     </row>
@@ -2891,7 +3585,7 @@
           <t>Months left</t>
         </is>
       </c>
-      <c r="B47" s="20" t="n">
+      <c r="B47" s="22" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2901,7 +3595,7 @@
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="B48" s="20">
+      <c r="B48" s="22">
         <f>B43-B45</f>
         <v/>
       </c>
@@ -2912,25 +3606,25 @@
           <t>Over (under) budget to date</t>
         </is>
       </c>
-      <c r="B49" s="20">
+      <c r="B49" s="22">
         <f>B45-B46</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="27" t="inlineStr">
+      <c r="A50" s="29" t="inlineStr">
         <is>
           <t>Over (under) budget, % of budget to date</t>
         </is>
       </c>
-      <c r="B50" s="31">
+      <c r="B50" s="33">
         <f>B45/B46-1</f>
         <v/>
       </c>
     </row>
     <row r="51"/>
     <row r="52">
-      <c r="A52" s="8" t="inlineStr">
+      <c r="A52" s="10" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
@@ -2964,13 +3658,13 @@
           <t>Jul 25</t>
         </is>
       </c>
-      <c r="B54" s="7" t="n">
+      <c r="B54" s="9" t="n">
         <v>17363</v>
       </c>
-      <c r="C54" s="7" t="n">
+      <c r="C54" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D54" s="9">
+      <c r="D54" s="11">
         <f>IF(C54=0,"",B54/C54)</f>
         <v/>
       </c>
@@ -2981,13 +3675,13 @@
           <t>Aug 25</t>
         </is>
       </c>
-      <c r="B55" s="7" t="n">
+      <c r="B55" s="9" t="n">
         <v>21144</v>
       </c>
-      <c r="C55" s="7" t="n">
+      <c r="C55" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D55" s="9">
+      <c r="D55" s="11">
         <f>IF(C55=0,"",B55/C55)</f>
         <v/>
       </c>
@@ -2998,13 +3692,13 @@
           <t>Sep 25</t>
         </is>
       </c>
-      <c r="B56" s="7" t="n">
+      <c r="B56" s="9" t="n">
         <v>17537</v>
       </c>
-      <c r="C56" s="7" t="n">
+      <c r="C56" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D56" s="9">
+      <c r="D56" s="11">
         <f>IF(C56=0,"",B56/C56)</f>
         <v/>
       </c>
@@ -3015,13 +3709,13 @@
           <t>Oct 25</t>
         </is>
       </c>
-      <c r="B57" s="7" t="n">
+      <c r="B57" s="9" t="n">
         <v>21925</v>
       </c>
-      <c r="C57" s="7" t="n">
+      <c r="C57" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D57" s="9">
+      <c r="D57" s="11">
         <f>IF(C57=0,"",B57/C57)</f>
         <v/>
       </c>
@@ -3032,13 +3726,13 @@
           <t>Nov 25</t>
         </is>
       </c>
-      <c r="B58" s="7" t="n">
+      <c r="B58" s="9" t="n">
         <v>21079</v>
       </c>
-      <c r="C58" s="7" t="n">
+      <c r="C58" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D58" s="9">
+      <c r="D58" s="11">
         <f>IF(C58=0,"",B58/C58)</f>
         <v/>
       </c>
@@ -3049,13 +3743,13 @@
           <t>Dec 25</t>
         </is>
       </c>
-      <c r="B59" s="7" t="n">
+      <c r="B59" s="9" t="n">
         <v>19272</v>
       </c>
-      <c r="C59" s="7" t="n">
+      <c r="C59" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D59" s="9">
+      <c r="D59" s="11">
         <f>IF(C59=0,"",B59/C59)</f>
         <v/>
       </c>
@@ -3066,13 +3760,13 @@
           <t>Jan 26</t>
         </is>
       </c>
-      <c r="B60" s="7" t="n">
+      <c r="B60" s="9" t="n">
         <v>21157</v>
       </c>
-      <c r="C60" s="7" t="n">
+      <c r="C60" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D60" s="9">
+      <c r="D60" s="11">
         <f>IF(C60=0,"",B60/C60)</f>
         <v/>
       </c>
@@ -3083,13 +3777,13 @@
           <t>Feb 26</t>
         </is>
       </c>
-      <c r="B61" s="7" t="n">
+      <c r="B61" s="9" t="n">
         <v>20743</v>
       </c>
-      <c r="C61" s="7" t="n">
+      <c r="C61" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D61" s="9">
+      <c r="D61" s="11">
         <f>IF(C61=0,"",B61/C61)</f>
         <v/>
       </c>
@@ -3100,13 +3794,13 @@
           <t>Mar 26</t>
         </is>
       </c>
-      <c r="B62" s="7" t="n">
+      <c r="B62" s="9" t="n">
         <v>16515</v>
       </c>
-      <c r="C62" s="7" t="n">
+      <c r="C62" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D62" s="9">
+      <c r="D62" s="11">
         <f>IF(C62=0,"",B62/C62)</f>
         <v/>
       </c>
@@ -3117,13 +3811,13 @@
           <t>Apr 26</t>
         </is>
       </c>
-      <c r="B63" s="7" t="n">
+      <c r="B63" s="9" t="n">
         <v>20451</v>
       </c>
-      <c r="C63" s="7" t="n">
+      <c r="C63" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D63" s="9">
+      <c r="D63" s="11">
         <f>IF(C63=0,"",B63/C63)</f>
         <v/>
       </c>
@@ -3134,13 +3828,13 @@
           <t>May 26</t>
         </is>
       </c>
-      <c r="B64" s="7" t="n">
+      <c r="B64" s="9" t="n">
         <v>21174</v>
       </c>
-      <c r="C64" s="7" t="n">
+      <c r="C64" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D64" s="9">
+      <c r="D64" s="11">
         <f>IF(C64=0,"",B64/C64)</f>
         <v/>
       </c>
@@ -3151,13 +3845,13 @@
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="B65" s="7" t="n">
+      <c r="B65" s="9" t="n">
         <v>20366</v>
       </c>
-      <c r="C65" s="7" t="n">
+      <c r="C65" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D65" s="9">
+      <c r="D65" s="11">
         <f>IF(C65=0,"",B65/C65)</f>
         <v/>
       </c>
@@ -3168,13 +3862,13 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B66" s="7" t="n">
+      <c r="B66" s="9" t="n">
         <v>23274</v>
       </c>
-      <c r="C66" s="7" t="n">
+      <c r="C66" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D66" s="9">
+      <c r="D66" s="11">
         <f>IF(C66=0,"",B66/C66)</f>
         <v/>
       </c>
@@ -3185,13 +3879,13 @@
           <t>Aug 26</t>
         </is>
       </c>
-      <c r="B67" s="7" t="n">
+      <c r="B67" s="9" t="n">
         <v>21500</v>
       </c>
-      <c r="C67" s="7" t="n">
+      <c r="C67" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D67" s="9">
+      <c r="D67" s="11">
         <f>IF(C67=0,"",B67/C67)</f>
         <v/>
       </c>
@@ -3202,32 +3896,32 @@
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B68" s="7" t="n">
+      <c r="B68" s="9" t="n">
         <v>22800</v>
       </c>
-      <c r="C68" s="7" t="n">
+      <c r="C68" s="9" t="n">
         <v>20000</v>
       </c>
-      <c r="D68" s="9">
+      <c r="D68" s="11">
         <f>IF(C68=0,"",B68/C68)</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="23" t="inlineStr">
+      <c r="A69" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B69" s="32">
+      <c r="B69" s="34">
         <f>SUM(B54:B68)</f>
         <v/>
       </c>
-      <c r="C69" s="32">
+      <c r="C69" s="34">
         <f>SUM(C54:C68)</f>
         <v/>
       </c>
-      <c r="D69" s="33">
+      <c r="D69" s="35">
         <f>IF(C69=0,"",B69/C69)</f>
         <v/>
       </c>
@@ -3235,14 +3929,14 @@
     <row r="70"/>
     <row r="71"/>
     <row r="72">
-      <c r="A72" s="25" t="inlineStr">
+      <c r="A72" s="27" t="inlineStr">
         <is>
           <t>Housing support</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="26" t="inlineStr">
+      <c r="A73" s="28" t="inlineStr">
         <is>
           <t>State Housing Program · $360,000 · Jan 2026 to Dec 2026</t>
         </is>
@@ -3262,7 +3956,7 @@
           <t>Grant total</t>
         </is>
       </c>
-      <c r="B75" s="20" t="n">
+      <c r="B75" s="22" t="n">
         <v>360000</v>
       </c>
     </row>
@@ -3272,7 +3966,7 @@
           <t>Received from the funder</t>
         </is>
       </c>
-      <c r="B76" s="20" t="n">
+      <c r="B76" s="22" t="n">
         <v>360000</v>
       </c>
     </row>
@@ -3282,7 +3976,7 @@
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="B77" s="20" t="n">
+      <c r="B77" s="22" t="n">
         <v>257700</v>
       </c>
     </row>
@@ -3292,7 +3986,7 @@
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="B78" s="20" t="n">
+      <c r="B78" s="22" t="n">
         <v>270000</v>
       </c>
     </row>
@@ -3302,7 +3996,7 @@
           <t>Months left</t>
         </is>
       </c>
-      <c r="B79" s="20" t="n">
+      <c r="B79" s="22" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3312,7 +4006,7 @@
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="B80" s="20">
+      <c r="B80" s="22">
         <f>B75-B77</f>
         <v/>
       </c>
@@ -3323,25 +4017,25 @@
           <t>Over (under) budget to date</t>
         </is>
       </c>
-      <c r="B81" s="20">
+      <c r="B81" s="22">
         <f>B77-B78</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="27" t="inlineStr">
+      <c r="A82" s="29" t="inlineStr">
         <is>
           <t>Over (under) budget, % of budget to date</t>
         </is>
       </c>
-      <c r="B82" s="31">
+      <c r="B82" s="33">
         <f>B77/B78-1</f>
         <v/>
       </c>
     </row>
     <row r="83"/>
     <row r="84">
-      <c r="A84" s="8" t="inlineStr">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
@@ -3375,13 +4069,13 @@
           <t>Jan 26</t>
         </is>
       </c>
-      <c r="B86" s="7" t="n">
+      <c r="B86" s="9" t="n">
         <v>30502</v>
       </c>
-      <c r="C86" s="7" t="n">
+      <c r="C86" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D86" s="9">
+      <c r="D86" s="11">
         <f>IF(C86=0,"",B86/C86)</f>
         <v/>
       </c>
@@ -3392,13 +4086,13 @@
           <t>Feb 26</t>
         </is>
       </c>
-      <c r="B87" s="7" t="n">
+      <c r="B87" s="9" t="n">
         <v>26508</v>
       </c>
-      <c r="C87" s="7" t="n">
+      <c r="C87" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D87" s="9">
+      <c r="D87" s="11">
         <f>IF(C87=0,"",B87/C87)</f>
         <v/>
       </c>
@@ -3409,13 +4103,13 @@
           <t>Mar 26</t>
         </is>
       </c>
-      <c r="B88" s="7" t="n">
+      <c r="B88" s="9" t="n">
         <v>24832</v>
       </c>
-      <c r="C88" s="7" t="n">
+      <c r="C88" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D88" s="9">
+      <c r="D88" s="11">
         <f>IF(C88=0,"",B88/C88)</f>
         <v/>
       </c>
@@ -3426,13 +4120,13 @@
           <t>Apr 26</t>
         </is>
       </c>
-      <c r="B89" s="7" t="n">
+      <c r="B89" s="9" t="n">
         <v>23730</v>
       </c>
-      <c r="C89" s="7" t="n">
+      <c r="C89" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D89" s="9">
+      <c r="D89" s="11">
         <f>IF(C89=0,"",B89/C89)</f>
         <v/>
       </c>
@@ -3443,13 +4137,13 @@
           <t>May 26</t>
         </is>
       </c>
-      <c r="B90" s="7" t="n">
+      <c r="B90" s="9" t="n">
         <v>31337</v>
       </c>
-      <c r="C90" s="7" t="n">
+      <c r="C90" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D90" s="9">
+      <c r="D90" s="11">
         <f>IF(C90=0,"",B90/C90)</f>
         <v/>
       </c>
@@ -3460,13 +4154,13 @@
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="B91" s="7" t="n">
+      <c r="B91" s="9" t="n">
         <v>29994</v>
       </c>
-      <c r="C91" s="7" t="n">
+      <c r="C91" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D91" s="9">
+      <c r="D91" s="11">
         <f>IF(C91=0,"",B91/C91)</f>
         <v/>
       </c>
@@ -3477,13 +4171,13 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B92" s="7" t="n">
+      <c r="B92" s="9" t="n">
         <v>29097</v>
       </c>
-      <c r="C92" s="7" t="n">
+      <c r="C92" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D92" s="9">
+      <c r="D92" s="11">
         <f>IF(C92=0,"",B92/C92)</f>
         <v/>
       </c>
@@ -3494,13 +4188,13 @@
           <t>Aug 26</t>
         </is>
       </c>
-      <c r="B93" s="7" t="n">
+      <c r="B93" s="9" t="n">
         <v>30500</v>
       </c>
-      <c r="C93" s="7" t="n">
+      <c r="C93" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D93" s="9">
+      <c r="D93" s="11">
         <f>IF(C93=0,"",B93/C93)</f>
         <v/>
       </c>
@@ -3511,32 +4205,32 @@
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B94" s="7" t="n">
+      <c r="B94" s="9" t="n">
         <v>31200</v>
       </c>
-      <c r="C94" s="7" t="n">
+      <c r="C94" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="D94" s="9">
+      <c r="D94" s="11">
         <f>IF(C94=0,"",B94/C94)</f>
         <v/>
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="23" t="inlineStr">
+      <c r="A95" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B95" s="32">
+      <c r="B95" s="34">
         <f>SUM(B86:B94)</f>
         <v/>
       </c>
-      <c r="C95" s="32">
+      <c r="C95" s="34">
         <f>SUM(C86:C94)</f>
         <v/>
       </c>
-      <c r="D95" s="33">
+      <c r="D95" s="35">
         <f>IF(C95=0,"",B95/C95)</f>
         <v/>
       </c>
@@ -3544,14 +4238,14 @@
     <row r="96"/>
     <row r="97"/>
     <row r="98">
-      <c r="A98" s="25" t="inlineStr">
+      <c r="A98" s="27" t="inlineStr">
         <is>
           <t>Mental health first aid</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="26" t="inlineStr">
+      <c r="A99" s="28" t="inlineStr">
         <is>
           <t>Federal health program · $120,000 · Apr 2026 to Mar 2027</t>
         </is>
@@ -3571,7 +4265,7 @@
           <t>Grant total</t>
         </is>
       </c>
-      <c r="B101" s="20" t="n">
+      <c r="B101" s="22" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -3581,7 +4275,7 @@
           <t>Received from the funder</t>
         </is>
       </c>
-      <c r="B102" s="20" t="n">
+      <c r="B102" s="22" t="n">
         <v>60000</v>
       </c>
     </row>
@@ -3591,7 +4285,7 @@
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="B103" s="20" t="n">
+      <c r="B103" s="22" t="n">
         <v>57200</v>
       </c>
     </row>
@@ -3601,7 +4295,7 @@
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="B104" s="20" t="n">
+      <c r="B104" s="22" t="n">
         <v>60000</v>
       </c>
     </row>
@@ -3611,7 +4305,7 @@
           <t>Months left</t>
         </is>
       </c>
-      <c r="B105" s="20" t="n">
+      <c r="B105" s="22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3621,7 +4315,7 @@
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="B106" s="20">
+      <c r="B106" s="22">
         <f>B101-B103</f>
         <v/>
       </c>
@@ -3632,25 +4326,25 @@
           <t>Over (under) budget to date</t>
         </is>
       </c>
-      <c r="B107" s="20">
+      <c r="B107" s="22">
         <f>B103-B104</f>
         <v/>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="27" t="inlineStr">
+      <c r="A108" s="29" t="inlineStr">
         <is>
           <t>Over (under) budget, % of budget to date</t>
         </is>
       </c>
-      <c r="B108" s="31">
+      <c r="B108" s="33">
         <f>B103/B104-1</f>
         <v/>
       </c>
     </row>
     <row r="109"/>
     <row r="110">
-      <c r="A110" s="8" t="inlineStr">
+      <c r="A110" s="10" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
@@ -3684,13 +4378,13 @@
           <t>Apr 26</t>
         </is>
       </c>
-      <c r="B112" s="7" t="n">
+      <c r="B112" s="9" t="n">
         <v>9584</v>
       </c>
-      <c r="C112" s="7" t="n">
+      <c r="C112" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="D112" s="9">
+      <c r="D112" s="11">
         <f>IF(C112=0,"",B112/C112)</f>
         <v/>
       </c>
@@ -3701,13 +4395,13 @@
           <t>May 26</t>
         </is>
       </c>
-      <c r="B113" s="7" t="n">
+      <c r="B113" s="9" t="n">
         <v>8950</v>
       </c>
-      <c r="C113" s="7" t="n">
+      <c r="C113" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="D113" s="9">
+      <c r="D113" s="11">
         <f>IF(C113=0,"",B113/C113)</f>
         <v/>
       </c>
@@ -3718,13 +4412,13 @@
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="B114" s="7" t="n">
+      <c r="B114" s="9" t="n">
         <v>9797</v>
       </c>
-      <c r="C114" s="7" t="n">
+      <c r="C114" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="D114" s="9">
+      <c r="D114" s="11">
         <f>IF(C114=0,"",B114/C114)</f>
         <v/>
       </c>
@@ -3735,13 +4429,13 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B115" s="7" t="n">
+      <c r="B115" s="9" t="n">
         <v>8669</v>
       </c>
-      <c r="C115" s="7" t="n">
+      <c r="C115" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="D115" s="9">
+      <c r="D115" s="11">
         <f>IF(C115=0,"",B115/C115)</f>
         <v/>
       </c>
@@ -3752,13 +4446,13 @@
           <t>Aug 26</t>
         </is>
       </c>
-      <c r="B116" s="7" t="n">
+      <c r="B116" s="9" t="n">
         <v>9400</v>
       </c>
-      <c r="C116" s="7" t="n">
+      <c r="C116" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="D116" s="9">
+      <c r="D116" s="11">
         <f>IF(C116=0,"",B116/C116)</f>
         <v/>
       </c>
@@ -3769,32 +4463,32 @@
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B117" s="7" t="n">
+      <c r="B117" s="9" t="n">
         <v>10800</v>
       </c>
-      <c r="C117" s="7" t="n">
+      <c r="C117" s="9" t="n">
         <v>10000</v>
       </c>
-      <c r="D117" s="9">
+      <c r="D117" s="11">
         <f>IF(C117=0,"",B117/C117)</f>
         <v/>
       </c>
     </row>
     <row r="118">
-      <c r="A118" s="23" t="inlineStr">
+      <c r="A118" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B118" s="32">
+      <c r="B118" s="34">
         <f>SUM(B112:B117)</f>
         <v/>
       </c>
-      <c r="C118" s="32">
+      <c r="C118" s="34">
         <f>SUM(C112:C117)</f>
         <v/>
       </c>
-      <c r="D118" s="33">
+      <c r="D118" s="35">
         <f>IF(C118=0,"",B118/C118)</f>
         <v/>
       </c>
@@ -3802,14 +4496,14 @@
     <row r="119"/>
     <row r="120"/>
     <row r="121">
-      <c r="A121" s="25" t="inlineStr">
+      <c r="A121" s="27" t="inlineStr">
         <is>
           <t>Digital literacy</t>
         </is>
       </c>
     </row>
     <row r="122">
-      <c r="A122" s="26" t="inlineStr">
+      <c r="A122" s="28" t="inlineStr">
         <is>
           <t>Philanthropic foundation · $90,000 · Oct 2025 to Mar 2027</t>
         </is>
@@ -3829,7 +4523,7 @@
           <t>Grant total</t>
         </is>
       </c>
-      <c r="B124" s="20" t="n">
+      <c r="B124" s="22" t="n">
         <v>90000</v>
       </c>
     </row>
@@ -3839,7 +4533,7 @@
           <t>Received from the funder</t>
         </is>
       </c>
-      <c r="B125" s="20" t="n">
+      <c r="B125" s="22" t="n">
         <v>45000</v>
       </c>
     </row>
@@ -3849,7 +4543,7 @@
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="B126" s="20" t="n">
+      <c r="B126" s="22" t="n">
         <v>59600</v>
       </c>
     </row>
@@ -3859,7 +4553,7 @@
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="B127" s="20" t="n">
+      <c r="B127" s="22" t="n">
         <v>60000</v>
       </c>
     </row>
@@ -3869,7 +4563,7 @@
           <t>Months left</t>
         </is>
       </c>
-      <c r="B128" s="20" t="n">
+      <c r="B128" s="22" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3879,7 +4573,7 @@
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="B129" s="20">
+      <c r="B129" s="22">
         <f>B124-B126</f>
         <v/>
       </c>
@@ -3890,25 +4584,25 @@
           <t>Over (under) budget to date</t>
         </is>
       </c>
-      <c r="B130" s="20">
+      <c r="B130" s="22">
         <f>B126-B127</f>
         <v/>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="27" t="inlineStr">
+      <c r="A131" s="29" t="inlineStr">
         <is>
           <t>Over (under) budget, % of budget to date</t>
         </is>
       </c>
-      <c r="B131" s="31">
+      <c r="B131" s="33">
         <f>B126/B127-1</f>
         <v/>
       </c>
     </row>
     <row r="132"/>
     <row r="133">
-      <c r="A133" s="8" t="inlineStr">
+      <c r="A133" s="10" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
@@ -3942,13 +4636,13 @@
           <t>Oct 25</t>
         </is>
       </c>
-      <c r="B135" s="7" t="n">
+      <c r="B135" s="9" t="n">
         <v>5160</v>
       </c>
-      <c r="C135" s="7" t="n">
+      <c r="C135" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D135" s="9">
+      <c r="D135" s="11">
         <f>IF(C135=0,"",B135/C135)</f>
         <v/>
       </c>
@@ -3959,13 +4653,13 @@
           <t>Nov 25</t>
         </is>
       </c>
-      <c r="B136" s="7" t="n">
+      <c r="B136" s="9" t="n">
         <v>4585</v>
       </c>
-      <c r="C136" s="7" t="n">
+      <c r="C136" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D136" s="9">
+      <c r="D136" s="11">
         <f>IF(C136=0,"",B136/C136)</f>
         <v/>
       </c>
@@ -3976,13 +4670,13 @@
           <t>Dec 25</t>
         </is>
       </c>
-      <c r="B137" s="7" t="n">
+      <c r="B137" s="9" t="n">
         <v>5221</v>
       </c>
-      <c r="C137" s="7" t="n">
+      <c r="C137" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D137" s="9">
+      <c r="D137" s="11">
         <f>IF(C137=0,"",B137/C137)</f>
         <v/>
       </c>
@@ -3993,13 +4687,13 @@
           <t>Jan 26</t>
         </is>
       </c>
-      <c r="B138" s="7" t="n">
+      <c r="B138" s="9" t="n">
         <v>4426</v>
       </c>
-      <c r="C138" s="7" t="n">
+      <c r="C138" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D138" s="9">
+      <c r="D138" s="11">
         <f>IF(C138=0,"",B138/C138)</f>
         <v/>
       </c>
@@ -4010,13 +4704,13 @@
           <t>Feb 26</t>
         </is>
       </c>
-      <c r="B139" s="7" t="n">
+      <c r="B139" s="9" t="n">
         <v>5408</v>
       </c>
-      <c r="C139" s="7" t="n">
+      <c r="C139" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D139" s="9">
+      <c r="D139" s="11">
         <f>IF(C139=0,"",B139/C139)</f>
         <v/>
       </c>
@@ -4027,13 +4721,13 @@
           <t>Mar 26</t>
         </is>
       </c>
-      <c r="B140" s="7" t="n">
+      <c r="B140" s="9" t="n">
         <v>5427</v>
       </c>
-      <c r="C140" s="7" t="n">
+      <c r="C140" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D140" s="9">
+      <c r="D140" s="11">
         <f>IF(C140=0,"",B140/C140)</f>
         <v/>
       </c>
@@ -4044,13 +4738,13 @@
           <t>Apr 26</t>
         </is>
       </c>
-      <c r="B141" s="7" t="n">
+      <c r="B141" s="9" t="n">
         <v>5509</v>
       </c>
-      <c r="C141" s="7" t="n">
+      <c r="C141" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D141" s="9">
+      <c r="D141" s="11">
         <f>IF(C141=0,"",B141/C141)</f>
         <v/>
       </c>
@@ -4061,13 +4755,13 @@
           <t>May 26</t>
         </is>
       </c>
-      <c r="B142" s="7" t="n">
+      <c r="B142" s="9" t="n">
         <v>4635</v>
       </c>
-      <c r="C142" s="7" t="n">
+      <c r="C142" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D142" s="9">
+      <c r="D142" s="11">
         <f>IF(C142=0,"",B142/C142)</f>
         <v/>
       </c>
@@ -4078,13 +4772,13 @@
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="B143" s="7" t="n">
+      <c r="B143" s="9" t="n">
         <v>4316</v>
       </c>
-      <c r="C143" s="7" t="n">
+      <c r="C143" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D143" s="9">
+      <c r="D143" s="11">
         <f>IF(C143=0,"",B143/C143)</f>
         <v/>
       </c>
@@ -4095,13 +4789,13 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B144" s="7" t="n">
+      <c r="B144" s="9" t="n">
         <v>4813</v>
       </c>
-      <c r="C144" s="7" t="n">
+      <c r="C144" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D144" s="9">
+      <c r="D144" s="11">
         <f>IF(C144=0,"",B144/C144)</f>
         <v/>
       </c>
@@ -4112,13 +4806,13 @@
           <t>Aug 26</t>
         </is>
       </c>
-      <c r="B145" s="7" t="n">
+      <c r="B145" s="9" t="n">
         <v>5200</v>
       </c>
-      <c r="C145" s="7" t="n">
+      <c r="C145" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D145" s="9">
+      <c r="D145" s="11">
         <f>IF(C145=0,"",B145/C145)</f>
         <v/>
       </c>
@@ -4129,32 +4823,32 @@
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B146" s="7" t="n">
+      <c r="B146" s="9" t="n">
         <v>4900</v>
       </c>
-      <c r="C146" s="7" t="n">
+      <c r="C146" s="9" t="n">
         <v>5000</v>
       </c>
-      <c r="D146" s="9">
+      <c r="D146" s="11">
         <f>IF(C146=0,"",B146/C146)</f>
         <v/>
       </c>
     </row>
     <row r="147">
-      <c r="A147" s="23" t="inlineStr">
+      <c r="A147" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B147" s="32">
+      <c r="B147" s="34">
         <f>SUM(B135:B146)</f>
         <v/>
       </c>
-      <c r="C147" s="32">
+      <c r="C147" s="34">
         <f>SUM(C135:C146)</f>
         <v/>
       </c>
-      <c r="D147" s="33">
+      <c r="D147" s="35">
         <f>IF(C147=0,"",B147/C147)</f>
         <v/>
       </c>
@@ -4162,14 +4856,14 @@
     <row r="148"/>
     <row r="149"/>
     <row r="150">
-      <c r="A150" s="25" t="inlineStr">
+      <c r="A150" s="27" t="inlineStr">
         <is>
           <t>Community meals</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" s="26" t="inlineStr">
+      <c r="A151" s="28" t="inlineStr">
         <is>
           <t>Local council community grant · $48,000 · Jul 2026 to Jun 2027</t>
         </is>
@@ -4189,7 +4883,7 @@
           <t>Grant total</t>
         </is>
       </c>
-      <c r="B153" s="20" t="n">
+      <c r="B153" s="22" t="n">
         <v>48000</v>
       </c>
     </row>
@@ -4199,7 +4893,7 @@
           <t>Received from the funder</t>
         </is>
       </c>
-      <c r="B154" s="20" t="n">
+      <c r="B154" s="22" t="n">
         <v>48000</v>
       </c>
     </row>
@@ -4209,7 +4903,7 @@
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="B155" s="20" t="n">
+      <c r="B155" s="22" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -4219,7 +4913,7 @@
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="B156" s="20" t="n">
+      <c r="B156" s="22" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -4229,7 +4923,7 @@
           <t>Months left</t>
         </is>
       </c>
-      <c r="B157" s="20" t="n">
+      <c r="B157" s="22" t="n">
         <v>9</v>
       </c>
     </row>
@@ -4239,7 +4933,7 @@
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="B158" s="20">
+      <c r="B158" s="22">
         <f>B153-B155</f>
         <v/>
       </c>
@@ -4250,25 +4944,25 @@
           <t>Over (under) budget to date</t>
         </is>
       </c>
-      <c r="B159" s="20">
+      <c r="B159" s="22">
         <f>B155-B156</f>
         <v/>
       </c>
     </row>
     <row r="160">
-      <c r="A160" s="27" t="inlineStr">
+      <c r="A160" s="29" t="inlineStr">
         <is>
           <t>Over (under) budget, % of budget to date</t>
         </is>
       </c>
-      <c r="B160" s="31">
+      <c r="B160" s="33">
         <f>B155/B156-1</f>
         <v/>
       </c>
     </row>
     <row r="161"/>
     <row r="162">
-      <c r="A162" s="8" t="inlineStr">
+      <c r="A162" s="10" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
@@ -4302,13 +4996,13 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B164" s="7" t="n">
+      <c r="B164" s="9" t="n">
         <v>3600</v>
       </c>
-      <c r="C164" s="7" t="n">
+      <c r="C164" s="9" t="n">
         <v>4000</v>
       </c>
-      <c r="D164" s="9">
+      <c r="D164" s="11">
         <f>IF(C164=0,"",B164/C164)</f>
         <v/>
       </c>
@@ -4319,13 +5013,13 @@
           <t>Aug 26</t>
         </is>
       </c>
-      <c r="B165" s="7" t="n">
+      <c r="B165" s="9" t="n">
         <v>4100</v>
       </c>
-      <c r="C165" s="7" t="n">
+      <c r="C165" s="9" t="n">
         <v>4000</v>
       </c>
-      <c r="D165" s="9">
+      <c r="D165" s="11">
         <f>IF(C165=0,"",B165/C165)</f>
         <v/>
       </c>
@@ -4336,32 +5030,32 @@
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B166" s="7" t="n">
+      <c r="B166" s="9" t="n">
         <v>4300</v>
       </c>
-      <c r="C166" s="7" t="n">
+      <c r="C166" s="9" t="n">
         <v>4000</v>
       </c>
-      <c r="D166" s="9">
+      <c r="D166" s="11">
         <f>IF(C166=0,"",B166/C166)</f>
         <v/>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="23" t="inlineStr">
+      <c r="A167" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B167" s="32">
+      <c r="B167" s="34">
         <f>SUM(B164:B166)</f>
         <v/>
       </c>
-      <c r="C167" s="32">
+      <c r="C167" s="34">
         <f>SUM(C164:C166)</f>
         <v/>
       </c>
-      <c r="D167" s="33">
+      <c r="D167" s="35">
         <f>IF(C167=0,"",B167/C167)</f>
         <v/>
       </c>
@@ -4369,14 +5063,14 @@
     <row r="168"/>
     <row r="169"/>
     <row r="170">
-      <c r="A170" s="25" t="inlineStr">
+      <c r="A170" s="27" t="inlineStr">
         <is>
           <t>Volunteer coordinator</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="26" t="inlineStr">
+      <c r="A171" s="28" t="inlineStr">
         <is>
           <t>State volunteering grant · $36,000 · Mar 2026 to Feb 2027</t>
         </is>
@@ -4396,7 +5090,7 @@
           <t>Grant total</t>
         </is>
       </c>
-      <c r="B173" s="20" t="n">
+      <c r="B173" s="22" t="n">
         <v>36000</v>
       </c>
     </row>
@@ -4406,7 +5100,7 @@
           <t>Received from the funder</t>
         </is>
       </c>
-      <c r="B174" s="20" t="n">
+      <c r="B174" s="22" t="n">
         <v>36000</v>
       </c>
     </row>
@@ -4416,7 +5110,7 @@
           <t>Spent to date</t>
         </is>
       </c>
-      <c r="B175" s="20" t="n">
+      <c r="B175" s="22" t="n">
         <v>21000</v>
       </c>
     </row>
@@ -4426,7 +5120,7 @@
           <t>Budget to date</t>
         </is>
       </c>
-      <c r="B176" s="20" t="n">
+      <c r="B176" s="22" t="n">
         <v>21000</v>
       </c>
     </row>
@@ -4436,7 +5130,7 @@
           <t>Months left</t>
         </is>
       </c>
-      <c r="B177" s="20" t="n">
+      <c r="B177" s="22" t="n">
         <v>5</v>
       </c>
     </row>
@@ -4446,7 +5140,7 @@
           <t>Still to spend</t>
         </is>
       </c>
-      <c r="B178" s="20">
+      <c r="B178" s="22">
         <f>B173-B175</f>
         <v/>
       </c>
@@ -4457,25 +5151,25 @@
           <t>Over (under) budget to date</t>
         </is>
       </c>
-      <c r="B179" s="20">
+      <c r="B179" s="22">
         <f>B175-B176</f>
         <v/>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="27" t="inlineStr">
+      <c r="A180" s="29" t="inlineStr">
         <is>
           <t>Over (under) budget, % of budget to date</t>
         </is>
       </c>
-      <c r="B180" s="31">
+      <c r="B180" s="33">
         <f>B175/B176-1</f>
         <v/>
       </c>
     </row>
     <row r="181"/>
     <row r="182">
-      <c r="A182" s="8" t="inlineStr">
+      <c r="A182" s="10" t="inlineStr">
         <is>
           <t>Spend by month against budget</t>
         </is>
@@ -4509,13 +5203,13 @@
           <t>Mar 26</t>
         </is>
       </c>
-      <c r="B184" s="7" t="n">
+      <c r="B184" s="9" t="n">
         <v>2932</v>
       </c>
-      <c r="C184" s="7" t="n">
+      <c r="C184" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D184" s="9">
+      <c r="D184" s="11">
         <f>IF(C184=0,"",B184/C184)</f>
         <v/>
       </c>
@@ -4526,13 +5220,13 @@
           <t>Apr 26</t>
         </is>
       </c>
-      <c r="B185" s="7" t="n">
+      <c r="B185" s="9" t="n">
         <v>3555</v>
       </c>
-      <c r="C185" s="7" t="n">
+      <c r="C185" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D185" s="9">
+      <c r="D185" s="11">
         <f>IF(C185=0,"",B185/C185)</f>
         <v/>
       </c>
@@ -4543,13 +5237,13 @@
           <t>May 26</t>
         </is>
       </c>
-      <c r="B186" s="7" t="n">
+      <c r="B186" s="9" t="n">
         <v>2649</v>
       </c>
-      <c r="C186" s="7" t="n">
+      <c r="C186" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D186" s="9">
+      <c r="D186" s="11">
         <f>IF(C186=0,"",B186/C186)</f>
         <v/>
       </c>
@@ -4560,13 +5254,13 @@
           <t>Jun 26</t>
         </is>
       </c>
-      <c r="B187" s="7" t="n">
+      <c r="B187" s="9" t="n">
         <v>2699</v>
       </c>
-      <c r="C187" s="7" t="n">
+      <c r="C187" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D187" s="9">
+      <c r="D187" s="11">
         <f>IF(C187=0,"",B187/C187)</f>
         <v/>
       </c>
@@ -4577,13 +5271,13 @@
           <t>Jul 26</t>
         </is>
       </c>
-      <c r="B188" s="7" t="n">
+      <c r="B188" s="9" t="n">
         <v>3165</v>
       </c>
-      <c r="C188" s="7" t="n">
+      <c r="C188" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D188" s="9">
+      <c r="D188" s="11">
         <f>IF(C188=0,"",B188/C188)</f>
         <v/>
       </c>
@@ -4594,13 +5288,13 @@
           <t>Aug 26</t>
         </is>
       </c>
-      <c r="B189" s="7" t="n">
+      <c r="B189" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="C189" s="7" t="n">
+      <c r="C189" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D189" s="9">
+      <c r="D189" s="11">
         <f>IF(C189=0,"",B189/C189)</f>
         <v/>
       </c>
@@ -4611,32 +5305,32 @@
           <t>Sep 26</t>
         </is>
       </c>
-      <c r="B190" s="7" t="n">
+      <c r="B190" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="C190" s="7" t="n">
+      <c r="C190" s="9" t="n">
         <v>3000</v>
       </c>
-      <c r="D190" s="9">
+      <c r="D190" s="11">
         <f>IF(C190=0,"",B190/C190)</f>
         <v/>
       </c>
     </row>
     <row r="191">
-      <c r="A191" s="23" t="inlineStr">
+      <c r="A191" s="25" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B191" s="32">
+      <c r="B191" s="34">
         <f>SUM(B184:B190)</f>
         <v/>
       </c>
-      <c r="C191" s="32">
+      <c r="C191" s="34">
         <f>SUM(C184:C190)</f>
         <v/>
       </c>
-      <c r="D191" s="33">
+      <c r="D191" s="35">
         <f>IF(C191=0,"",B191/C191)</f>
         <v/>
       </c>
@@ -4650,7 +5344,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4691,56 +5385,56 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet</t>
+          <t>Sample Community Services Ltd · SAMPLE DATA (invented) · The Fourth Sheet · Made with Python (openpyxl)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026)</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
         </is>
       </c>
     </row>
     <row r="4"/>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>The organisation</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="36" t="inlineStr">
         <is>
           <t>What it is</t>
         </is>
       </c>
-      <c r="B6" s="35" t="inlineStr">
+      <c r="B6" s="37" t="inlineStr">
         <is>
           <t>A Brisbane community services charity funded by six grants, donations, events and program fees. About 18 staff. Registered charity, income-tax exempt.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="34" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>Reporting month</t>
         </is>
       </c>
-      <c r="B7" s="35" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>September 2026, compared with August 2026</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="34" t="inlineStr">
+      <c r="A8" s="36" t="inlineStr">
         <is>
           <t>Financial year</t>
         </is>
       </c>
-      <c r="B8" s="35" t="inlineStr">
+      <c r="B8" s="37" t="inlineStr">
         <is>
           <t>FY2027: 1 July 2026 to 30 June 2027</t>
         </is>
@@ -4748,103 +5442,103 @@
     </row>
     <row r="9"/>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Grants</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="34" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>Youth outreach</t>
         </is>
       </c>
-      <c r="B11" s="35" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>State Department of Families: $480,000, 2025-07 to 2027-06</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="34" t="inlineStr">
+      <c r="A12" s="36" t="inlineStr">
         <is>
           <t>Housing support</t>
         </is>
       </c>
-      <c r="B12" s="35" t="inlineStr">
+      <c r="B12" s="37" t="inlineStr">
         <is>
           <t>State Housing Program: $360,000, 2026-01 to 2026-12</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="34" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>Community meals</t>
         </is>
       </c>
-      <c r="B13" s="35" t="inlineStr">
+      <c r="B13" s="37" t="inlineStr">
         <is>
           <t>Local council community grant: $48,000, 2026-07 to 2027-06</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
         <is>
           <t>Digital literacy</t>
         </is>
       </c>
-      <c r="B14" s="35" t="inlineStr">
+      <c r="B14" s="37" t="inlineStr">
         <is>
           <t>Philanthropic foundation: $90,000, 2025-10 to 2027-03</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="34" t="inlineStr">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>Mental health first aid</t>
         </is>
       </c>
-      <c r="B15" s="35" t="inlineStr">
+      <c r="B15" s="37" t="inlineStr">
         <is>
           <t>Federal health program: $120,000, 2026-04 to 2027-03</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="34" t="inlineStr">
+      <c r="A16" s="36" t="inlineStr">
         <is>
           <t>Volunteer coordinator</t>
         </is>
       </c>
-      <c r="B16" s="35" t="inlineStr">
+      <c r="B16" s="37" t="inlineStr">
         <is>
           <t>State volunteering grant: $36,000, 2026-03 to 2027-02</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="34" t="inlineStr">
+      <c r="A17" s="36" t="inlineStr">
         <is>
           <t>Grant income</t>
         </is>
       </c>
-      <c r="B17" s="35" t="inlineStr">
+      <c r="B17" s="37" t="inlineStr">
         <is>
           <t>recognised as the money is spent on the program</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="34" t="inlineStr">
+      <c r="A18" s="36" t="inlineStr">
         <is>
           <t>Unspent grants</t>
         </is>
       </c>
-      <c r="B18" s="35" t="inlineStr">
+      <c r="B18" s="37" t="inlineStr">
         <is>
           <t>instalments received but not yet spent are a liability (grants received in advance)</t>
         </is>
@@ -4852,55 +5546,55 @@
     </row>
     <row r="19"/>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Other income and costs</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="34" t="inlineStr">
+      <c r="A21" s="36" t="inlineStr">
         <is>
           <t>Donations</t>
         </is>
       </c>
-      <c r="B21" s="35" t="inlineStr">
+      <c r="B21" s="37" t="inlineStr">
         <is>
           <t>including the spring appeal in September</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="34" t="inlineStr">
+      <c r="A22" s="36" t="inlineStr">
         <is>
           <t>Fundraising event</t>
         </is>
       </c>
-      <c r="B22" s="35" t="inlineStr">
+      <c r="B22" s="37" t="inlineStr">
         <is>
           <t>September gala: income and costs in the same month</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="34" t="inlineStr">
+      <c r="A23" s="36" t="inlineStr">
         <is>
           <t>Grant-funded spending</t>
         </is>
       </c>
-      <c r="B23" s="35" t="inlineStr">
+      <c r="B23" s="37" t="inlineStr">
         <is>
           <t>75% wages, the rest program costs</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="34" t="inlineStr">
+      <c r="A24" s="36" t="inlineStr">
         <is>
           <t>Income tax</t>
         </is>
       </c>
-      <c r="B24" s="35" t="inlineStr">
+      <c r="B24" s="37" t="inlineStr">
         <is>
           <t>none: registered charity, income-tax exempt</t>
         </is>
@@ -4908,67 +5602,67 @@
     </row>
     <row r="25"/>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Cash and balance sheet</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="34" t="inlineStr">
+      <c r="A27" s="36" t="inlineStr">
         <is>
           <t>Suppliers</t>
         </is>
       </c>
-      <c r="B27" s="35" t="inlineStr">
+      <c r="B27" s="37" t="inlineStr">
         <is>
           <t>paid the following month</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="34" t="inlineStr">
+      <c r="A28" s="36" t="inlineStr">
         <is>
           <t>Unrestricted cash</t>
         </is>
       </c>
-      <c r="B28" s="35" t="inlineStr">
+      <c r="B28" s="37" t="inlineStr">
         <is>
           <t>cash at bank less unspent grant money</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="34" t="inlineStr">
+      <c r="A29" s="36" t="inlineStr">
         <is>
           <t>Cash runway</t>
         </is>
       </c>
-      <c r="B29" s="35" t="inlineStr">
+      <c r="B29" s="37" t="inlineStr">
         <is>
           <t>unrestricted cash ÷ this month's cash spending</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="34" t="inlineStr">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Reserves target</t>
         </is>
       </c>
-      <c r="B30" s="35" t="inlineStr">
+      <c r="B30" s="37" t="inlineStr">
         <is>
           <t>3 months of spending</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="34" t="inlineStr">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>GST</t>
         </is>
       </c>
-      <c r="B31" s="35" t="inlineStr">
+      <c r="B31" s="37" t="inlineStr">
         <is>
           <t>excluded throughout, for simplicity</t>
         </is>
@@ -4976,7 +5670,7 @@
     </row>
     <row r="32"/>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Checks (all passed)</t>
         </is>
@@ -5024,8 +5718,9 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Print check (done before this file was saved)</t>
         </is>
@@ -5086,7 +5781,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>

<commit_message>
Budget colours: over red, under green, within 1% amber (site, PDF, Excel, PowerPoint, board table)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/nfp-sample-statements.xlsx
+++ b/media/exports/nfp-sample-statements.xlsx
@@ -384,28 +384,14 @@
             </spPr>
           </dPt>
           <dPt>
-            <idx val="1"/>
+            <idx val="3"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="B42318"/>
+                <a:srgbClr val="8A6D3B"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:solidFill>
-                  <a:srgbClr val="B42318"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </dPt>
-          <dPt>
-            <idx val="2"/>
-            <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="B42318"/>
-              </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:solidFill>
-                  <a:srgbClr val="B42318"/>
+                  <a:srgbClr val="8A6D3B"/>
                 </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -962,7 +948,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1036,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Spending to date against budget to date (the grant spread evenly over its months). Over or under budget in red; within 1% in amber.</t>
+          <t>Spending to date against budget to date (the grant spread evenly over its months). Over budget in red, under budget in green; within 1% in amber.</t>
         </is>
       </c>
     </row>
@@ -1179,7 +1165,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1221,7 +1207,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1954,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2012,7 +1998,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2280,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2335,7 +2321,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -2689,7 +2675,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2739,7 +2725,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -3141,7 +3127,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3186,7 +3172,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5330,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5392,7 +5378,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:35am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:34am</t>
         </is>
       </c>
     </row>
@@ -5781,7 +5767,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Community Services Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:35am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 nfp-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:34am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>